<commit_message>
Results: Regularized Classifier Comparison (Full Dataset, Fixed -Col bug)
</commit_message>
<xml_diff>
--- a/classification_results/regularized/comprehensive_results.xlsx
+++ b/classification_results/regularized/comprehensive_results.xlsx
@@ -515,34 +515,34 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.9</v>
+        <v>0.8833333333333334</v>
       </c>
       <c r="D2" t="n">
-        <v>0.0816496580927726</v>
+        <v>0.08498365855987973</v>
       </c>
       <c r="E2" t="n">
-        <v>0.9666666666666666</v>
+        <v>0.9708333333333334</v>
       </c>
       <c r="F2" t="n">
-        <v>0.06666666666666654</v>
+        <v>0.08750000000000002</v>
       </c>
       <c r="G2" t="n">
-        <v>0.95625</v>
+        <v>0.95</v>
       </c>
       <c r="H2" t="n">
-        <v>0.03750000000000001</v>
+        <v>0.04677071733467426</v>
       </c>
       <c r="I2" t="n">
-        <v>0.8006349206349206</v>
+        <v>0.7792063492063492</v>
       </c>
       <c r="J2" t="n">
-        <v>0.2070892711811676</v>
+        <v>0.2056719043154454</v>
       </c>
       <c r="K2" t="n">
-        <v>0.96</v>
+        <v>0.9099999999999999</v>
       </c>
       <c r="L2" t="n">
-        <v>0.07999999999999999</v>
+        <v>0.1113552872566004</v>
       </c>
       <c r="M2" t="n">
         <v>0.75</v>
@@ -569,10 +569,10 @@
         <v>0.05270462766947298</v>
       </c>
       <c r="E3" t="n">
-        <v>0.9458333333333334</v>
+        <v>0.95</v>
       </c>
       <c r="F3" t="n">
-        <v>0.02916666666666679</v>
+        <v>0.03333333333333333</v>
       </c>
       <c r="G3" t="n">
         <v>0.975</v>
@@ -623,10 +623,10 @@
         <v>0.08333333333333337</v>
       </c>
       <c r="G4" t="n">
-        <v>0.99375</v>
+        <v>0.9875</v>
       </c>
       <c r="H4" t="n">
-        <v>0.0125</v>
+        <v>0.025</v>
       </c>
       <c r="I4" t="n">
         <v>0.8806349206349207</v>
@@ -710,37 +710,37 @@
         <v>0.6</v>
       </c>
       <c r="D6" t="n">
-        <v>0.08970695222838923</v>
+        <v>0.05756395979652219</v>
       </c>
       <c r="E6" t="n">
-        <v>0.9</v>
+        <v>0.9076923076923078</v>
       </c>
       <c r="F6" t="n">
-        <v>0.3</v>
+        <v>0.3076923076923078</v>
       </c>
       <c r="G6" t="n">
-        <v>0.6555555555555556</v>
+        <v>0.6500000000000001</v>
       </c>
       <c r="H6" t="n">
-        <v>0.06712803318663652</v>
+        <v>0.09229582069908975</v>
       </c>
       <c r="I6" t="n">
-        <v>0.7373205741626794</v>
+        <v>0.7433857370699476</v>
       </c>
       <c r="J6" t="n">
-        <v>0.06788460360499277</v>
+        <v>0.04414718906103555</v>
       </c>
       <c r="K6" t="n">
-        <v>0.6711888111888112</v>
+        <v>0.6663403263403262</v>
       </c>
       <c r="L6" t="n">
-        <v>0.04626475337406512</v>
+        <v>0.02684990915472382</v>
       </c>
       <c r="M6" t="n">
-        <v>0.8222222222222222</v>
+        <v>0.8444444444444444</v>
       </c>
       <c r="N6" t="n">
-        <v>0.1133115447465063</v>
+        <v>0.08888888888888888</v>
       </c>
     </row>
     <row r="7">
@@ -755,40 +755,40 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.6615384615384615</v>
+        <v>0.6461538461538462</v>
       </c>
       <c r="D7" t="n">
-        <v>0.07844645405527362</v>
+        <v>0.06153846153846153</v>
       </c>
       <c r="E7" t="n">
         <v>0.7538461538461538</v>
       </c>
       <c r="F7" t="n">
-        <v>0.09230769230769231</v>
+        <v>0.1076923076923076</v>
       </c>
       <c r="G7" t="n">
-        <v>0.5833333333333333</v>
+        <v>0.5833333333333334</v>
       </c>
       <c r="H7" t="n">
-        <v>0.1082977149423218</v>
+        <v>0.09781564923143894</v>
       </c>
       <c r="I7" t="n">
-        <v>0.7844383686488949</v>
+        <v>0.7715728715728716</v>
       </c>
       <c r="J7" t="n">
-        <v>0.04968673265970842</v>
+        <v>0.04058360428882864</v>
       </c>
       <c r="K7" t="n">
-        <v>0.7045221445221446</v>
+        <v>0.7000777000777001</v>
       </c>
       <c r="L7" t="n">
-        <v>0.05632303646484361</v>
+        <v>0.04901637209756619</v>
       </c>
       <c r="M7" t="n">
-        <v>0.888888888888889</v>
+        <v>0.8666666666666666</v>
       </c>
       <c r="N7" t="n">
-        <v>0.07027283689263066</v>
+        <v>0.08314794192830979</v>
       </c>
     </row>
     <row r="8">
@@ -803,40 +803,40 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.6000000000000001</v>
+        <v>0.6307692307692307</v>
       </c>
       <c r="D8" t="n">
-        <v>0.07536891516255932</v>
+        <v>0.07536891516255934</v>
       </c>
       <c r="E8" t="n">
-        <v>0.9153846153846154</v>
+        <v>0.9461538461538461</v>
       </c>
       <c r="F8" t="n">
-        <v>0.3153846153846153</v>
+        <v>0.3153846153846154</v>
       </c>
       <c r="G8" t="n">
-        <v>0.5944444444444443</v>
+        <v>0.5444444444444445</v>
       </c>
       <c r="H8" t="n">
-        <v>0.1486565351139961</v>
+        <v>0.1507184440694504</v>
       </c>
       <c r="I8" t="n">
-        <v>0.7272416334955034</v>
+        <v>0.7456060606060607</v>
       </c>
       <c r="J8" t="n">
-        <v>0.05691230061863263</v>
+        <v>0.08278940945388297</v>
       </c>
       <c r="K8" t="n">
-        <v>0.6887878787878787</v>
+        <v>0.6985680985680986</v>
       </c>
       <c r="L8" t="n">
-        <v>0.0523953327189115</v>
+        <v>0.02081867374915897</v>
       </c>
       <c r="M8" t="n">
-        <v>0.7777777777777777</v>
+        <v>0.8222222222222222</v>
       </c>
       <c r="N8" t="n">
-        <v>0.09938079899999065</v>
+        <v>0.180534186769688</v>
       </c>
     </row>
     <row r="9">
@@ -851,40 +851,40 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.5846153846153845</v>
+        <v>0.6153846153846153</v>
       </c>
       <c r="D9" t="n">
-        <v>0.06153846153846154</v>
+        <v>0.04865042554105199</v>
       </c>
       <c r="E9" t="n">
         <v>0.9076923076923077</v>
       </c>
       <c r="F9" t="n">
-        <v>0.3230769230769232</v>
+        <v>0.2923076923076924</v>
       </c>
       <c r="G9" t="n">
-        <v>0.5388888888888889</v>
+        <v>0.5333333333333333</v>
       </c>
       <c r="H9" t="n">
-        <v>0.1119413426644993</v>
+        <v>0.1130388330520878</v>
       </c>
       <c r="I9" t="n">
-        <v>0.7293506493506493</v>
+        <v>0.7557666894509</v>
       </c>
       <c r="J9" t="n">
-        <v>0.05404248277019266</v>
+        <v>0.03857217572392534</v>
       </c>
       <c r="K9" t="n">
-        <v>0.6596736596736597</v>
+        <v>0.6724009324009323</v>
       </c>
       <c r="L9" t="n">
-        <v>0.02121084040294139</v>
+        <v>0.02246080112117707</v>
       </c>
       <c r="M9" t="n">
-        <v>0.8222222222222222</v>
+        <v>0.8666666666666666</v>
       </c>
       <c r="N9" t="n">
-        <v>0.1133115447465063</v>
+        <v>0.08314794192830979</v>
       </c>
     </row>
     <row r="10">
@@ -902,7 +902,7 @@
         <v>0.7555555555555554</v>
       </c>
       <c r="D10" t="n">
-        <v>0.12957670877434</v>
+        <v>0.1632993161855452</v>
       </c>
       <c r="E10" t="n">
         <v>0.9777777777777779</v>
@@ -911,28 +911,28 @@
         <v>0.2222222222222224</v>
       </c>
       <c r="G10" t="n">
-        <v>0.82</v>
+        <v>0.8099999999999999</v>
       </c>
       <c r="H10" t="n">
-        <v>0.10295630140987</v>
+        <v>0.1019803902718557</v>
       </c>
       <c r="I10" t="n">
-        <v>0.7199134199134198</v>
+        <v>0.7354689754689755</v>
       </c>
       <c r="J10" t="n">
-        <v>0.1474126090770152</v>
+        <v>0.1664586421894694</v>
       </c>
       <c r="K10" t="n">
-        <v>0.8166666666666668</v>
+        <v>0.8066666666666666</v>
       </c>
       <c r="L10" t="n">
-        <v>0.1855921454276674</v>
+        <v>0.2194943684420577</v>
       </c>
       <c r="M10" t="n">
-        <v>0.67</v>
+        <v>0.71</v>
       </c>
       <c r="N10" t="n">
-        <v>0.1886796226411321</v>
+        <v>0.1907878402833891</v>
       </c>
     </row>
     <row r="11">
@@ -947,16 +947,16 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.6666666666666667</v>
+        <v>0.6888888888888889</v>
       </c>
       <c r="D11" t="n">
-        <v>0.1721325931647741</v>
+        <v>0.1777777777777778</v>
       </c>
       <c r="E11" t="n">
-        <v>0.9111111111111111</v>
+        <v>0.9166666666666666</v>
       </c>
       <c r="F11" t="n">
-        <v>0.2444444444444444</v>
+        <v>0.2277777777777777</v>
       </c>
       <c r="G11" t="n">
         <v>0.77</v>
@@ -965,22 +965,22 @@
         <v>0.198997487421324</v>
       </c>
       <c r="I11" t="n">
-        <v>0.6433333333333333</v>
+        <v>0.67</v>
       </c>
       <c r="J11" t="n">
-        <v>0.2012737218593404</v>
+        <v>0.2111871208194288</v>
       </c>
       <c r="K11" t="n">
-        <v>0.6833333333333333</v>
+        <v>0.6933333333333334</v>
       </c>
       <c r="L11" t="n">
-        <v>0.2438123139721299</v>
+        <v>0.247341419454522</v>
       </c>
       <c r="M11" t="n">
-        <v>0.64</v>
+        <v>0.6799999999999999</v>
       </c>
       <c r="N11" t="n">
-        <v>0.2437211521390788</v>
+        <v>0.2501999200639361</v>
       </c>
     </row>
     <row r="12">
@@ -998,37 +998,37 @@
         <v>0.8222222222222222</v>
       </c>
       <c r="D12" t="n">
-        <v>0.1133115447465063</v>
+        <v>0.05443310539518171</v>
       </c>
       <c r="E12" t="n">
-        <v>0.9888888888888889</v>
+        <v>0.9944444444444445</v>
       </c>
       <c r="F12" t="n">
-        <v>0.1666666666666667</v>
+        <v>0.1722222222222223</v>
       </c>
       <c r="G12" t="n">
-        <v>0.86</v>
+        <v>0.8699999999999999</v>
       </c>
       <c r="H12" t="n">
-        <v>0.09695359714832659</v>
+        <v>0.116619037896906</v>
       </c>
       <c r="I12" t="n">
-        <v>0.7980952380952381</v>
+        <v>0.8025396825396826</v>
       </c>
       <c r="J12" t="n">
-        <v>0.1255410061202597</v>
+        <v>0.07604218372865965</v>
       </c>
       <c r="K12" t="n">
-        <v>0.8833333333333332</v>
+        <v>0.8933333333333333</v>
       </c>
       <c r="L12" t="n">
-        <v>0.1452966314513558</v>
+        <v>0.1372750685464934</v>
       </c>
       <c r="M12" t="n">
         <v>0.77</v>
       </c>
       <c r="N12" t="n">
-        <v>0.2039607805437114</v>
+        <v>0.16</v>
       </c>
     </row>
     <row r="13">
@@ -1125,10 +1125,10 @@
         <v>0.9166666666666666</v>
       </c>
       <c r="C2" t="n">
-        <v>0.6666666666666667</v>
+        <v>0.6888888888888889</v>
       </c>
       <c r="D2" t="n">
-        <v>0.6615384615384615</v>
+        <v>0.6461538461538462</v>
       </c>
     </row>
     <row r="3">
@@ -1144,7 +1144,7 @@
         <v>0.8222222222222222</v>
       </c>
       <c r="D3" t="n">
-        <v>0.6000000000000001</v>
+        <v>0.6307692307692307</v>
       </c>
     </row>
     <row r="4">
@@ -1154,7 +1154,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.9</v>
+        <v>0.8833333333333334</v>
       </c>
       <c r="C4" t="n">
         <v>0.7555555555555554</v>
@@ -1176,7 +1176,7 @@
         <v>0.7777777777777777</v>
       </c>
       <c r="D5" t="n">
-        <v>0.5846153846153845</v>
+        <v>0.6153846153846153</v>
       </c>
     </row>
   </sheetData>
@@ -1225,10 +1225,10 @@
         <v>0.8706349206349205</v>
       </c>
       <c r="C2" t="n">
-        <v>0.6433333333333333</v>
+        <v>0.67</v>
       </c>
       <c r="D2" t="n">
-        <v>0.7844383686488949</v>
+        <v>0.7715728715728716</v>
       </c>
     </row>
     <row r="3">
@@ -1241,10 +1241,10 @@
         <v>0.8806349206349207</v>
       </c>
       <c r="C3" t="n">
-        <v>0.7980952380952381</v>
+        <v>0.8025396825396826</v>
       </c>
       <c r="D3" t="n">
-        <v>0.7272416334955034</v>
+        <v>0.7456060606060607</v>
       </c>
     </row>
     <row r="4">
@@ -1254,13 +1254,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.8006349206349206</v>
+        <v>0.7792063492063492</v>
       </c>
       <c r="C4" t="n">
-        <v>0.7199134199134198</v>
+        <v>0.7354689754689755</v>
       </c>
       <c r="D4" t="n">
-        <v>0.7373205741626794</v>
+        <v>0.7433857370699476</v>
       </c>
     </row>
     <row r="5">
@@ -1276,7 +1276,7 @@
         <v>0.7042857142857143</v>
       </c>
       <c r="D5" t="n">
-        <v>0.7293506493506493</v>
+        <v>0.7557666894509</v>
       </c>
     </row>
   </sheetData>
@@ -1328,7 +1328,7 @@
         <v>0.77</v>
       </c>
       <c r="D2" t="n">
-        <v>0.5833333333333333</v>
+        <v>0.5833333333333334</v>
       </c>
     </row>
     <row r="3">
@@ -1338,13 +1338,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.99375</v>
+        <v>0.9875</v>
       </c>
       <c r="C3" t="n">
-        <v>0.86</v>
+        <v>0.8699999999999999</v>
       </c>
       <c r="D3" t="n">
-        <v>0.5944444444444443</v>
+        <v>0.5444444444444445</v>
       </c>
     </row>
     <row r="4">
@@ -1354,13 +1354,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.95625</v>
+        <v>0.95</v>
       </c>
       <c r="C4" t="n">
-        <v>0.82</v>
+        <v>0.8099999999999999</v>
       </c>
       <c r="D4" t="n">
-        <v>0.6555555555555556</v>
+        <v>0.6500000000000001</v>
       </c>
     </row>
     <row r="5">
@@ -1376,7 +1376,7 @@
         <v>0.8699999999999999</v>
       </c>
       <c r="D5" t="n">
-        <v>0.5388888888888889</v>
+        <v>0.5333333333333333</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Final: Classification using Raw_Final.csv (No Circularity, Full Dataset 190 cells)
</commit_message>
<xml_diff>
--- a/classification_results/regularized/comprehensive_results.xlsx
+++ b/classification_results/regularized/comprehensive_results.xlsx
@@ -515,40 +515,40 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.8833333333333334</v>
+        <v>0.7894736842105263</v>
       </c>
       <c r="D2" t="n">
-        <v>0.08498365855987973</v>
+        <v>0.0941502306315701</v>
       </c>
       <c r="E2" t="n">
-        <v>0.9708333333333334</v>
+        <v>0.9447368421052632</v>
       </c>
       <c r="F2" t="n">
-        <v>0.08750000000000002</v>
+        <v>0.1552631578947369</v>
       </c>
       <c r="G2" t="n">
-        <v>0.95</v>
+        <v>0.8733333333333333</v>
       </c>
       <c r="H2" t="n">
-        <v>0.04677071733467426</v>
+        <v>0.07118052168020879</v>
       </c>
       <c r="I2" t="n">
-        <v>0.7792063492063492</v>
+        <v>0.7783969728242173</v>
       </c>
       <c r="J2" t="n">
-        <v>0.2056719043154454</v>
+        <v>0.09499268341627182</v>
       </c>
       <c r="K2" t="n">
-        <v>0.9099999999999999</v>
+        <v>0.7827777777777778</v>
       </c>
       <c r="L2" t="n">
-        <v>0.1113552872566004</v>
+        <v>0.1044444444444444</v>
       </c>
       <c r="M2" t="n">
-        <v>0.75</v>
+        <v>0.7777777777777777</v>
       </c>
       <c r="N2" t="n">
-        <v>0.273861278752583</v>
+        <v>0.09938079899999065</v>
       </c>
     </row>
     <row r="3">
@@ -563,40 +563,40 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.9166666666666666</v>
+        <v>0.8631578947368421</v>
       </c>
       <c r="D3" t="n">
-        <v>0.05270462766947298</v>
+        <v>0.04210526315789474</v>
       </c>
       <c r="E3" t="n">
-        <v>0.95</v>
+        <v>0.881578947368421</v>
       </c>
       <c r="F3" t="n">
-        <v>0.03333333333333333</v>
+        <v>0.01842105263157889</v>
       </c>
       <c r="G3" t="n">
-        <v>0.975</v>
+        <v>0.8777777777777779</v>
       </c>
       <c r="H3" t="n">
-        <v>0.05</v>
+        <v>0.08491099188685688</v>
       </c>
       <c r="I3" t="n">
-        <v>0.8706349206349205</v>
+        <v>0.8617543859649123</v>
       </c>
       <c r="J3" t="n">
-        <v>0.07998173134821665</v>
+        <v>0.0358009384228472</v>
       </c>
       <c r="K3" t="n">
-        <v>0.9099999999999999</v>
+        <v>0.8387878787878786</v>
       </c>
       <c r="L3" t="n">
-        <v>0.1113552872566004</v>
+        <v>0.06552932503503284</v>
       </c>
       <c r="M3" t="n">
-        <v>0.85</v>
+        <v>0.888888888888889</v>
       </c>
       <c r="N3" t="n">
-        <v>0.1224744871391589</v>
+        <v>1.110223024625157e-16</v>
       </c>
     </row>
     <row r="4">
@@ -611,40 +611,40 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.9166666666666666</v>
+        <v>0.8421052631578947</v>
       </c>
       <c r="D4" t="n">
-        <v>0.05270462766947298</v>
+        <v>0.04707511531578504</v>
       </c>
       <c r="E4" t="n">
-        <v>1</v>
+        <v>0.9894736842105264</v>
       </c>
       <c r="F4" t="n">
-        <v>0.08333333333333337</v>
+        <v>0.1473684210526317</v>
       </c>
       <c r="G4" t="n">
-        <v>0.9875</v>
+        <v>0.9133333333333333</v>
       </c>
       <c r="H4" t="n">
-        <v>0.025</v>
+        <v>0.07993824777157758</v>
       </c>
       <c r="I4" t="n">
-        <v>0.8806349206349207</v>
+        <v>0.8439766081871344</v>
       </c>
       <c r="J4" t="n">
-        <v>0.06621464291801239</v>
+        <v>0.03976332979813007</v>
       </c>
       <c r="K4" t="n">
-        <v>0.8933333333333333</v>
+        <v>0.8064646464646466</v>
       </c>
       <c r="L4" t="n">
-        <v>0.1372750685464934</v>
+        <v>0.07234918556961416</v>
       </c>
       <c r="M4" t="n">
-        <v>0.9</v>
+        <v>0.888888888888889</v>
       </c>
       <c r="N4" t="n">
-        <v>0.1224744871391589</v>
+        <v>1.110223024625157e-16</v>
       </c>
     </row>
     <row r="5">
@@ -659,40 +659,40 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.8833333333333332</v>
+        <v>0.7789473684210526</v>
       </c>
       <c r="D5" t="n">
-        <v>0.08498365855987973</v>
+        <v>0.06982367979695579</v>
       </c>
       <c r="E5" t="n">
-        <v>0.9875</v>
+        <v>0.9289473684210525</v>
       </c>
       <c r="F5" t="n">
-        <v>0.1041666666666669</v>
+        <v>0.1499999999999999</v>
       </c>
       <c r="G5" t="n">
-        <v>0.98125</v>
+        <v>0.8266666666666665</v>
       </c>
       <c r="H5" t="n">
-        <v>0.025</v>
+        <v>0.1041366623454221</v>
       </c>
       <c r="I5" t="n">
-        <v>0.7892063492063492</v>
+        <v>0.7823809523809524</v>
       </c>
       <c r="J5" t="n">
-        <v>0.205223793066532</v>
+        <v>0.06693144697452993</v>
       </c>
       <c r="K5" t="n">
-        <v>0.8933333333333333</v>
+        <v>0.7411255411255412</v>
       </c>
       <c r="L5" t="n">
-        <v>0.1372750685464934</v>
+        <v>0.08498090206193512</v>
       </c>
       <c r="M5" t="n">
-        <v>0.8</v>
+        <v>0.8444444444444444</v>
       </c>
       <c r="N5" t="n">
-        <v>0.291547594742265</v>
+        <v>0.1133115447465063</v>
       </c>
     </row>
     <row r="6">
@@ -707,40 +707,40 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.6</v>
+        <v>0.5777777777777777</v>
       </c>
       <c r="D6" t="n">
-        <v>0.05756395979652219</v>
+        <v>0.1030402055055078</v>
       </c>
       <c r="E6" t="n">
-        <v>0.9076923076923078</v>
+        <v>0.9444444444444444</v>
       </c>
       <c r="F6" t="n">
-        <v>0.3076923076923078</v>
+        <v>0.3666666666666667</v>
       </c>
       <c r="G6" t="n">
-        <v>0.6500000000000001</v>
+        <v>0.6320987654320988</v>
       </c>
       <c r="H6" t="n">
-        <v>0.09229582069908975</v>
+        <v>0.1182610371834868</v>
       </c>
       <c r="I6" t="n">
-        <v>0.7433857370699476</v>
+        <v>0.5445793972109761</v>
       </c>
       <c r="J6" t="n">
-        <v>0.04414718906103555</v>
+        <v>0.1490446170454986</v>
       </c>
       <c r="K6" t="n">
-        <v>0.6663403263403262</v>
+        <v>0.5777777777777777</v>
       </c>
       <c r="L6" t="n">
-        <v>0.02684990915472382</v>
+        <v>0.1030402055055078</v>
       </c>
       <c r="M6" t="n">
-        <v>0.8444444444444444</v>
+        <v>0.5333333333333334</v>
       </c>
       <c r="N6" t="n">
-        <v>0.08888888888888888</v>
+        <v>0.1777777777777778</v>
       </c>
     </row>
     <row r="7">
@@ -755,40 +755,40 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.6461538461538462</v>
+        <v>0.5777777777777778</v>
       </c>
       <c r="D7" t="n">
-        <v>0.06153846153846153</v>
+        <v>0.05665577237325316</v>
       </c>
       <c r="E7" t="n">
-        <v>0.7538461538461538</v>
+        <v>0.7583333333333333</v>
       </c>
       <c r="F7" t="n">
-        <v>0.1076923076923076</v>
+        <v>0.1805555555555555</v>
       </c>
       <c r="G7" t="n">
-        <v>0.5833333333333334</v>
+        <v>0.5456790123456791</v>
       </c>
       <c r="H7" t="n">
-        <v>0.09781564923143894</v>
+        <v>0.06957532248694008</v>
       </c>
       <c r="I7" t="n">
-        <v>0.7715728715728716</v>
+        <v>0.5738588896483632</v>
       </c>
       <c r="J7" t="n">
-        <v>0.04058360428882864</v>
+        <v>0.100569593215003</v>
       </c>
       <c r="K7" t="n">
-        <v>0.7000777000777001</v>
+        <v>0.5741880341880343</v>
       </c>
       <c r="L7" t="n">
-        <v>0.04901637209756619</v>
+        <v>0.04214429294012985</v>
       </c>
       <c r="M7" t="n">
-        <v>0.8666666666666666</v>
+        <v>0.6</v>
       </c>
       <c r="N7" t="n">
-        <v>0.08314794192830979</v>
+        <v>0.180534186769688</v>
       </c>
     </row>
     <row r="8">
@@ -803,40 +803,40 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.6307692307692307</v>
+        <v>0.5666666666666667</v>
       </c>
       <c r="D8" t="n">
-        <v>0.07536891516255934</v>
+        <v>0.06478835438717</v>
       </c>
       <c r="E8" t="n">
-        <v>0.9461538461538461</v>
+        <v>0.986111111111111</v>
       </c>
       <c r="F8" t="n">
-        <v>0.3153846153846154</v>
+        <v>0.4194444444444444</v>
       </c>
       <c r="G8" t="n">
-        <v>0.5444444444444445</v>
+        <v>0.6271604938271605</v>
       </c>
       <c r="H8" t="n">
-        <v>0.1507184440694504</v>
+        <v>0.09317512229191705</v>
       </c>
       <c r="I8" t="n">
-        <v>0.7456060606060607</v>
+        <v>0.5518954248366013</v>
       </c>
       <c r="J8" t="n">
-        <v>0.08278940945388297</v>
+        <v>0.1058691188372695</v>
       </c>
       <c r="K8" t="n">
-        <v>0.6985680985680986</v>
+        <v>0.5611111111111111</v>
       </c>
       <c r="L8" t="n">
-        <v>0.02081867374915897</v>
+        <v>0.06186404847588912</v>
       </c>
       <c r="M8" t="n">
-        <v>0.8222222222222222</v>
+        <v>0.5555555555555556</v>
       </c>
       <c r="N8" t="n">
-        <v>0.180534186769688</v>
+        <v>0.1571348402636772</v>
       </c>
     </row>
     <row r="9">
@@ -851,40 +851,40 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.6153846153846153</v>
+        <v>0.5444444444444445</v>
       </c>
       <c r="D9" t="n">
-        <v>0.04865042554105199</v>
+        <v>0.0816496580927726</v>
       </c>
       <c r="E9" t="n">
-        <v>0.9076923076923077</v>
+        <v>0.9527777777777778</v>
       </c>
       <c r="F9" t="n">
-        <v>0.2923076923076924</v>
+        <v>0.4083333333333333</v>
       </c>
       <c r="G9" t="n">
-        <v>0.5333333333333333</v>
+        <v>0.5950617283950617</v>
       </c>
       <c r="H9" t="n">
-        <v>0.1130388330520878</v>
+        <v>0.09447469861584686</v>
       </c>
       <c r="I9" t="n">
-        <v>0.7557666894509</v>
+        <v>0.5116939407341883</v>
       </c>
       <c r="J9" t="n">
-        <v>0.03857217572392534</v>
+        <v>0.1444145070927954</v>
       </c>
       <c r="K9" t="n">
-        <v>0.6724009324009323</v>
+        <v>0.5272727272727272</v>
       </c>
       <c r="L9" t="n">
-        <v>0.02246080112117707</v>
+        <v>0.08351770238440617</v>
       </c>
       <c r="M9" t="n">
-        <v>0.8666666666666666</v>
+        <v>0.5111111111111111</v>
       </c>
       <c r="N9" t="n">
-        <v>0.08314794192830979</v>
+        <v>0.193728841935141</v>
       </c>
     </row>
     <row r="10">
@@ -902,7 +902,7 @@
         <v>0.7555555555555554</v>
       </c>
       <c r="D10" t="n">
-        <v>0.1632993161855452</v>
+        <v>0.12957670877434</v>
       </c>
       <c r="E10" t="n">
         <v>0.9777777777777779</v>
@@ -911,28 +911,28 @@
         <v>0.2222222222222224</v>
       </c>
       <c r="G10" t="n">
-        <v>0.8099999999999999</v>
+        <v>0.82</v>
       </c>
       <c r="H10" t="n">
-        <v>0.1019803902718557</v>
+        <v>0.10295630140987</v>
       </c>
       <c r="I10" t="n">
-        <v>0.7354689754689755</v>
+        <v>0.7199134199134198</v>
       </c>
       <c r="J10" t="n">
-        <v>0.1664586421894694</v>
+        <v>0.1474126090770152</v>
       </c>
       <c r="K10" t="n">
-        <v>0.8066666666666666</v>
+        <v>0.8166666666666668</v>
       </c>
       <c r="L10" t="n">
-        <v>0.2194943684420577</v>
+        <v>0.1855921454276674</v>
       </c>
       <c r="M10" t="n">
-        <v>0.71</v>
+        <v>0.67</v>
       </c>
       <c r="N10" t="n">
-        <v>0.1907878402833891</v>
+        <v>0.1886796226411321</v>
       </c>
     </row>
     <row r="11">
@@ -947,16 +947,16 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.6888888888888889</v>
+        <v>0.6666666666666667</v>
       </c>
       <c r="D11" t="n">
-        <v>0.1777777777777778</v>
+        <v>0.1721325931647741</v>
       </c>
       <c r="E11" t="n">
-        <v>0.9166666666666666</v>
+        <v>0.9111111111111111</v>
       </c>
       <c r="F11" t="n">
-        <v>0.2277777777777777</v>
+        <v>0.2444444444444444</v>
       </c>
       <c r="G11" t="n">
         <v>0.77</v>
@@ -965,22 +965,22 @@
         <v>0.198997487421324</v>
       </c>
       <c r="I11" t="n">
-        <v>0.67</v>
+        <v>0.6433333333333333</v>
       </c>
       <c r="J11" t="n">
-        <v>0.2111871208194288</v>
+        <v>0.2012737218593404</v>
       </c>
       <c r="K11" t="n">
-        <v>0.6933333333333334</v>
+        <v>0.6833333333333333</v>
       </c>
       <c r="L11" t="n">
-        <v>0.247341419454522</v>
+        <v>0.2438123139721299</v>
       </c>
       <c r="M11" t="n">
-        <v>0.6799999999999999</v>
+        <v>0.64</v>
       </c>
       <c r="N11" t="n">
-        <v>0.2501999200639361</v>
+        <v>0.2437211521390788</v>
       </c>
     </row>
     <row r="12">
@@ -998,37 +998,37 @@
         <v>0.8222222222222222</v>
       </c>
       <c r="D12" t="n">
-        <v>0.05443310539518171</v>
+        <v>0.1133115447465063</v>
       </c>
       <c r="E12" t="n">
-        <v>0.9944444444444445</v>
+        <v>0.9888888888888889</v>
       </c>
       <c r="F12" t="n">
-        <v>0.1722222222222223</v>
+        <v>0.1666666666666667</v>
       </c>
       <c r="G12" t="n">
-        <v>0.8699999999999999</v>
+        <v>0.86</v>
       </c>
       <c r="H12" t="n">
-        <v>0.116619037896906</v>
+        <v>0.09695359714832659</v>
       </c>
       <c r="I12" t="n">
-        <v>0.8025396825396826</v>
+        <v>0.7980952380952381</v>
       </c>
       <c r="J12" t="n">
-        <v>0.07604218372865965</v>
+        <v>0.1255410061202597</v>
       </c>
       <c r="K12" t="n">
-        <v>0.8933333333333333</v>
+        <v>0.8833333333333332</v>
       </c>
       <c r="L12" t="n">
-        <v>0.1372750685464934</v>
+        <v>0.1452966314513558</v>
       </c>
       <c r="M12" t="n">
         <v>0.77</v>
       </c>
       <c r="N12" t="n">
-        <v>0.16</v>
+        <v>0.2039607805437114</v>
       </c>
     </row>
     <row r="13">
@@ -1122,13 +1122,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.9166666666666666</v>
+        <v>0.8631578947368421</v>
       </c>
       <c r="C2" t="n">
-        <v>0.6888888888888889</v>
+        <v>0.6666666666666667</v>
       </c>
       <c r="D2" t="n">
-        <v>0.6461538461538462</v>
+        <v>0.5777777777777778</v>
       </c>
     </row>
     <row r="3">
@@ -1138,13 +1138,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.9166666666666666</v>
+        <v>0.8421052631578947</v>
       </c>
       <c r="C3" t="n">
         <v>0.8222222222222222</v>
       </c>
       <c r="D3" t="n">
-        <v>0.6307692307692307</v>
+        <v>0.5666666666666667</v>
       </c>
     </row>
     <row r="4">
@@ -1154,13 +1154,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.8833333333333334</v>
+        <v>0.7894736842105263</v>
       </c>
       <c r="C4" t="n">
         <v>0.7555555555555554</v>
       </c>
       <c r="D4" t="n">
-        <v>0.6</v>
+        <v>0.5777777777777777</v>
       </c>
     </row>
     <row r="5">
@@ -1170,13 +1170,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.8833333333333332</v>
+        <v>0.7789473684210526</v>
       </c>
       <c r="C5" t="n">
         <v>0.7777777777777777</v>
       </c>
       <c r="D5" t="n">
-        <v>0.6153846153846153</v>
+        <v>0.5444444444444445</v>
       </c>
     </row>
   </sheetData>
@@ -1222,13 +1222,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.8706349206349205</v>
+        <v>0.8617543859649123</v>
       </c>
       <c r="C2" t="n">
-        <v>0.67</v>
+        <v>0.6433333333333333</v>
       </c>
       <c r="D2" t="n">
-        <v>0.7715728715728716</v>
+        <v>0.5738588896483632</v>
       </c>
     </row>
     <row r="3">
@@ -1238,13 +1238,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.8806349206349207</v>
+        <v>0.8439766081871344</v>
       </c>
       <c r="C3" t="n">
-        <v>0.8025396825396826</v>
+        <v>0.7980952380952381</v>
       </c>
       <c r="D3" t="n">
-        <v>0.7456060606060607</v>
+        <v>0.5518954248366013</v>
       </c>
     </row>
     <row r="4">
@@ -1254,13 +1254,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.7792063492063492</v>
+        <v>0.7783969728242173</v>
       </c>
       <c r="C4" t="n">
-        <v>0.7354689754689755</v>
+        <v>0.7199134199134198</v>
       </c>
       <c r="D4" t="n">
-        <v>0.7433857370699476</v>
+        <v>0.5445793972109761</v>
       </c>
     </row>
     <row r="5">
@@ -1270,13 +1270,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.7892063492063492</v>
+        <v>0.7823809523809524</v>
       </c>
       <c r="C5" t="n">
         <v>0.7042857142857143</v>
       </c>
       <c r="D5" t="n">
-        <v>0.7557666894509</v>
+        <v>0.5116939407341883</v>
       </c>
     </row>
   </sheetData>
@@ -1322,13 +1322,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.975</v>
+        <v>0.8777777777777779</v>
       </c>
       <c r="C2" t="n">
         <v>0.77</v>
       </c>
       <c r="D2" t="n">
-        <v>0.5833333333333334</v>
+        <v>0.5456790123456791</v>
       </c>
     </row>
     <row r="3">
@@ -1338,13 +1338,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.9875</v>
+        <v>0.9133333333333333</v>
       </c>
       <c r="C3" t="n">
-        <v>0.8699999999999999</v>
+        <v>0.86</v>
       </c>
       <c r="D3" t="n">
-        <v>0.5444444444444445</v>
+        <v>0.6271604938271605</v>
       </c>
     </row>
     <row r="4">
@@ -1354,13 +1354,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.95</v>
+        <v>0.8733333333333333</v>
       </c>
       <c r="C4" t="n">
-        <v>0.8099999999999999</v>
+        <v>0.82</v>
       </c>
       <c r="D4" t="n">
-        <v>0.6500000000000001</v>
+        <v>0.6320987654320988</v>
       </c>
     </row>
     <row r="5">
@@ -1370,13 +1370,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.98125</v>
+        <v>0.8266666666666665</v>
       </c>
       <c r="C5" t="n">
         <v>0.8699999999999999</v>
       </c>
       <c r="D5" t="n">
-        <v>0.5333333333333333</v>
+        <v>0.5950617283950617</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Final Fix: Added DMSO support to collagen extraction, achieving full 200 cell dataset
</commit_message>
<xml_diff>
--- a/classification_results/regularized/comprehensive_results.xlsx
+++ b/classification_results/regularized/comprehensive_results.xlsx
@@ -515,40 +515,40 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.7894736842105263</v>
+        <v>0.7684210526315789</v>
       </c>
       <c r="D2" t="n">
-        <v>0.0941502306315701</v>
+        <v>0.09761703679469162</v>
       </c>
       <c r="E2" t="n">
         <v>0.9447368421052632</v>
       </c>
       <c r="F2" t="n">
-        <v>0.1552631578947369</v>
+        <v>0.1763157894736843</v>
       </c>
       <c r="G2" t="n">
-        <v>0.8733333333333333</v>
+        <v>0.8666666666666666</v>
       </c>
       <c r="H2" t="n">
-        <v>0.07118052168020879</v>
+        <v>0.07027283689263066</v>
       </c>
       <c r="I2" t="n">
-        <v>0.7783969728242173</v>
+        <v>0.7658479532163742</v>
       </c>
       <c r="J2" t="n">
-        <v>0.09499268341627182</v>
+        <v>0.09998570398136811</v>
       </c>
       <c r="K2" t="n">
-        <v>0.7827777777777778</v>
+        <v>0.7365656565656564</v>
       </c>
       <c r="L2" t="n">
-        <v>0.1044444444444444</v>
+        <v>0.1008451177889093</v>
       </c>
       <c r="M2" t="n">
-        <v>0.7777777777777777</v>
+        <v>0.7999999999999999</v>
       </c>
       <c r="N2" t="n">
-        <v>0.09938079899999065</v>
+        <v>0.1088662107903635</v>
       </c>
     </row>
     <row r="3">
@@ -563,34 +563,34 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.8631578947368421</v>
+        <v>0.8736842105263157</v>
       </c>
       <c r="D3" t="n">
         <v>0.04210526315789474</v>
       </c>
       <c r="E3" t="n">
-        <v>0.881578947368421</v>
+        <v>0.8842105263157893</v>
       </c>
       <c r="F3" t="n">
-        <v>0.01842105263157889</v>
+        <v>0.01052631578947361</v>
       </c>
       <c r="G3" t="n">
-        <v>0.8777777777777779</v>
+        <v>0.8822222222222222</v>
       </c>
       <c r="H3" t="n">
-        <v>0.08491099188685688</v>
+        <v>0.08680899993166491</v>
       </c>
       <c r="I3" t="n">
-        <v>0.8617543859649123</v>
+        <v>0.8711111111111111</v>
       </c>
       <c r="J3" t="n">
-        <v>0.0358009384228472</v>
+        <v>0.03555555555555552</v>
       </c>
       <c r="K3" t="n">
-        <v>0.8387878787878786</v>
+        <v>0.8565656565656565</v>
       </c>
       <c r="L3" t="n">
-        <v>0.06552932503503284</v>
+        <v>0.06464646464646462</v>
       </c>
       <c r="M3" t="n">
         <v>0.888888888888889</v>
@@ -611,40 +611,40 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.8421052631578947</v>
+        <v>0.8315789473684211</v>
       </c>
       <c r="D4" t="n">
-        <v>0.04707511531578504</v>
+        <v>0.03938586722919937</v>
       </c>
       <c r="E4" t="n">
-        <v>0.9894736842105264</v>
+        <v>0.9921052631578948</v>
       </c>
       <c r="F4" t="n">
-        <v>0.1473684210526317</v>
+        <v>0.1605263157894737</v>
       </c>
       <c r="G4" t="n">
-        <v>0.9133333333333333</v>
+        <v>0.9066666666666666</v>
       </c>
       <c r="H4" t="n">
-        <v>0.07993824777157758</v>
+        <v>0.08508528764034064</v>
       </c>
       <c r="I4" t="n">
-        <v>0.8439766081871344</v>
+        <v>0.8309047127622978</v>
       </c>
       <c r="J4" t="n">
-        <v>0.03976332979813007</v>
+        <v>0.03302185523827871</v>
       </c>
       <c r="K4" t="n">
-        <v>0.8064646464646466</v>
+        <v>0.8036868686868687</v>
       </c>
       <c r="L4" t="n">
-        <v>0.07234918556961416</v>
+        <v>0.06933510216481169</v>
       </c>
       <c r="M4" t="n">
-        <v>0.888888888888889</v>
+        <v>0.8666666666666666</v>
       </c>
       <c r="N4" t="n">
-        <v>1.110223024625157e-16</v>
+        <v>0.04444444444444442</v>
       </c>
     </row>
     <row r="5">
@@ -707,34 +707,34 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.5777777777777777</v>
+        <v>0.5888888888888889</v>
       </c>
       <c r="D6" t="n">
-        <v>0.1030402055055078</v>
+        <v>0.06666666666666667</v>
       </c>
       <c r="E6" t="n">
-        <v>0.9444444444444444</v>
+        <v>0.9472222222222222</v>
       </c>
       <c r="F6" t="n">
-        <v>0.3666666666666667</v>
+        <v>0.3583333333333333</v>
       </c>
       <c r="G6" t="n">
-        <v>0.6320987654320988</v>
+        <v>0.6419753086419753</v>
       </c>
       <c r="H6" t="n">
-        <v>0.1182610371834868</v>
+        <v>0.1050471475860871</v>
       </c>
       <c r="I6" t="n">
-        <v>0.5445793972109761</v>
+        <v>0.5473684210526316</v>
       </c>
       <c r="J6" t="n">
-        <v>0.1490446170454986</v>
+        <v>0.1279940493127902</v>
       </c>
       <c r="K6" t="n">
-        <v>0.5777777777777777</v>
+        <v>0.6066666666666667</v>
       </c>
       <c r="L6" t="n">
-        <v>0.1030402055055078</v>
+        <v>0.06347936380926975</v>
       </c>
       <c r="M6" t="n">
         <v>0.5333333333333334</v>
@@ -767,10 +767,10 @@
         <v>0.1805555555555555</v>
       </c>
       <c r="G7" t="n">
-        <v>0.5456790123456791</v>
+        <v>0.5530864197530864</v>
       </c>
       <c r="H7" t="n">
-        <v>0.06957532248694008</v>
+        <v>0.07784633466881205</v>
       </c>
       <c r="I7" t="n">
         <v>0.5738588896483632</v>
@@ -803,40 +803,40 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.5666666666666667</v>
+        <v>0.6555555555555556</v>
       </c>
       <c r="D8" t="n">
-        <v>0.06478835438717</v>
+        <v>0.06478835438716998</v>
       </c>
       <c r="E8" t="n">
-        <v>0.986111111111111</v>
+        <v>0.9805555555555555</v>
       </c>
       <c r="F8" t="n">
-        <v>0.4194444444444444</v>
+        <v>0.325</v>
       </c>
       <c r="G8" t="n">
-        <v>0.6271604938271605</v>
+        <v>0.6814814814814816</v>
       </c>
       <c r="H8" t="n">
-        <v>0.09317512229191705</v>
+        <v>0.1068882015896956</v>
       </c>
       <c r="I8" t="n">
-        <v>0.5518954248366013</v>
+        <v>0.6575271512113616</v>
       </c>
       <c r="J8" t="n">
-        <v>0.1058691188372695</v>
+        <v>0.09466974295331763</v>
       </c>
       <c r="K8" t="n">
-        <v>0.5611111111111111</v>
+        <v>0.6450505050505051</v>
       </c>
       <c r="L8" t="n">
-        <v>0.06186404847588912</v>
+        <v>0.04906887313546757</v>
       </c>
       <c r="M8" t="n">
-        <v>0.5555555555555556</v>
+        <v>0.6888888888888889</v>
       </c>
       <c r="N8" t="n">
-        <v>0.1571348402636772</v>
+        <v>0.1632993161855452</v>
       </c>
     </row>
     <row r="9">
@@ -857,16 +857,16 @@
         <v>0.0816496580927726</v>
       </c>
       <c r="E9" t="n">
-        <v>0.9527777777777778</v>
+        <v>0.9555555555555555</v>
       </c>
       <c r="F9" t="n">
-        <v>0.4083333333333333</v>
+        <v>0.411111111111111</v>
       </c>
       <c r="G9" t="n">
-        <v>0.5950617283950617</v>
+        <v>0.5975308641975309</v>
       </c>
       <c r="H9" t="n">
-        <v>0.09447469861584686</v>
+        <v>0.09802189254952696</v>
       </c>
       <c r="I9" t="n">
         <v>0.5116939407341883</v>
@@ -899,40 +899,40 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0.7555555555555554</v>
+        <v>0.7777777777777778</v>
       </c>
       <c r="D10" t="n">
-        <v>0.12957670877434</v>
+        <v>0.1571348402636772</v>
       </c>
       <c r="E10" t="n">
-        <v>0.9777777777777779</v>
+        <v>0.9944444444444445</v>
       </c>
       <c r="F10" t="n">
-        <v>0.2222222222222224</v>
+        <v>0.2166666666666667</v>
       </c>
       <c r="G10" t="n">
-        <v>0.82</v>
+        <v>0.8600000000000001</v>
       </c>
       <c r="H10" t="n">
-        <v>0.10295630140987</v>
+        <v>0.1067707825203131</v>
       </c>
       <c r="I10" t="n">
-        <v>0.7199134199134198</v>
+        <v>0.762063492063492</v>
       </c>
       <c r="J10" t="n">
-        <v>0.1474126090770152</v>
+        <v>0.1645905461167204</v>
       </c>
       <c r="K10" t="n">
-        <v>0.8166666666666668</v>
+        <v>0.7833333333333333</v>
       </c>
       <c r="L10" t="n">
-        <v>0.1855921454276674</v>
+        <v>0.19436506316151</v>
       </c>
       <c r="M10" t="n">
-        <v>0.67</v>
+        <v>0.76</v>
       </c>
       <c r="N10" t="n">
-        <v>0.1886796226411321</v>
+        <v>0.1593737745050923</v>
       </c>
     </row>
     <row r="11">
@@ -947,40 +947,40 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.6666666666666667</v>
+        <v>0.6444444444444445</v>
       </c>
       <c r="D11" t="n">
-        <v>0.1721325931647741</v>
+        <v>0.257240820062005</v>
       </c>
       <c r="E11" t="n">
-        <v>0.9111111111111111</v>
+        <v>0.888888888888889</v>
       </c>
       <c r="F11" t="n">
-        <v>0.2444444444444444</v>
+        <v>0.2444444444444445</v>
       </c>
       <c r="G11" t="n">
-        <v>0.77</v>
+        <v>0.75</v>
       </c>
       <c r="H11" t="n">
-        <v>0.198997487421324</v>
+        <v>0.1949358868961793</v>
       </c>
       <c r="I11" t="n">
-        <v>0.6433333333333333</v>
+        <v>0.611111111111111</v>
       </c>
       <c r="J11" t="n">
-        <v>0.2012737218593404</v>
+        <v>0.2533723166886974</v>
       </c>
       <c r="K11" t="n">
-        <v>0.6833333333333333</v>
+        <v>0.6933333333333334</v>
       </c>
       <c r="L11" t="n">
-        <v>0.2438123139721299</v>
+        <v>0.2969474326842678</v>
       </c>
       <c r="M11" t="n">
-        <v>0.64</v>
+        <v>0.58</v>
       </c>
       <c r="N11" t="n">
-        <v>0.2437211521390788</v>
+        <v>0.2657066051117284</v>
       </c>
     </row>
     <row r="12">
@@ -995,40 +995,40 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0.8222222222222222</v>
+        <v>0.7777777777777777</v>
       </c>
       <c r="D12" t="n">
-        <v>0.1133115447465063</v>
+        <v>0.1217161238900369</v>
       </c>
       <c r="E12" t="n">
-        <v>0.9888888888888889</v>
+        <v>1</v>
       </c>
       <c r="F12" t="n">
-        <v>0.1666666666666667</v>
+        <v>0.2222222222222223</v>
       </c>
       <c r="G12" t="n">
-        <v>0.86</v>
+        <v>0.8800000000000001</v>
       </c>
       <c r="H12" t="n">
-        <v>0.09695359714832659</v>
+        <v>0.08124038404635961</v>
       </c>
       <c r="I12" t="n">
-        <v>0.7980952380952381</v>
+        <v>0.7676190476190476</v>
       </c>
       <c r="J12" t="n">
-        <v>0.1255410061202597</v>
+        <v>0.1447619047619048</v>
       </c>
       <c r="K12" t="n">
-        <v>0.8833333333333332</v>
+        <v>0.7466666666666667</v>
       </c>
       <c r="L12" t="n">
-        <v>0.1452966314513558</v>
+        <v>0.1423610433604175</v>
       </c>
       <c r="M12" t="n">
-        <v>0.77</v>
+        <v>0.8099999999999999</v>
       </c>
       <c r="N12" t="n">
-        <v>0.2039607805437114</v>
+        <v>0.1854723699099141</v>
       </c>
     </row>
     <row r="13">
@@ -1046,37 +1046,37 @@
         <v>0.7777777777777777</v>
       </c>
       <c r="D13" t="n">
-        <v>0.1217161238900369</v>
+        <v>0.1987615979999813</v>
       </c>
       <c r="E13" t="n">
-        <v>0.9388888888888889</v>
+        <v>0.9722222222222223</v>
       </c>
       <c r="F13" t="n">
-        <v>0.1611111111111112</v>
+        <v>0.1944444444444446</v>
       </c>
       <c r="G13" t="n">
         <v>0.8699999999999999</v>
       </c>
       <c r="H13" t="n">
-        <v>0.1077032961426901</v>
+        <v>0.09797958971132713</v>
       </c>
       <c r="I13" t="n">
-        <v>0.7042857142857143</v>
+        <v>0.7244444444444443</v>
       </c>
       <c r="J13" t="n">
-        <v>0.204420534932381</v>
+        <v>0.2504711609529843</v>
       </c>
       <c r="K13" t="n">
-        <v>0.8433333333333334</v>
+        <v>0.8400000000000001</v>
       </c>
       <c r="L13" t="n">
-        <v>0.1348249894410446</v>
+        <v>0.233238075793812</v>
       </c>
       <c r="M13" t="n">
-        <v>0.6599999999999999</v>
+        <v>0.71</v>
       </c>
       <c r="N13" t="n">
-        <v>0.2596150997149434</v>
+        <v>0.2939387691339814</v>
       </c>
     </row>
   </sheetData>
@@ -1122,10 +1122,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.8631578947368421</v>
+        <v>0.8736842105263157</v>
       </c>
       <c r="C2" t="n">
-        <v>0.6666666666666667</v>
+        <v>0.6444444444444445</v>
       </c>
       <c r="D2" t="n">
         <v>0.5777777777777778</v>
@@ -1138,13 +1138,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.8421052631578947</v>
+        <v>0.8315789473684211</v>
       </c>
       <c r="C3" t="n">
-        <v>0.8222222222222222</v>
+        <v>0.7777777777777777</v>
       </c>
       <c r="D3" t="n">
-        <v>0.5666666666666667</v>
+        <v>0.6555555555555556</v>
       </c>
     </row>
     <row r="4">
@@ -1154,13 +1154,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.7894736842105263</v>
+        <v>0.7684210526315789</v>
       </c>
       <c r="C4" t="n">
-        <v>0.7555555555555554</v>
+        <v>0.7777777777777778</v>
       </c>
       <c r="D4" t="n">
-        <v>0.5777777777777777</v>
+        <v>0.5888888888888889</v>
       </c>
     </row>
     <row r="5">
@@ -1222,10 +1222,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.8617543859649123</v>
+        <v>0.8711111111111111</v>
       </c>
       <c r="C2" t="n">
-        <v>0.6433333333333333</v>
+        <v>0.611111111111111</v>
       </c>
       <c r="D2" t="n">
         <v>0.5738588896483632</v>
@@ -1238,13 +1238,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.8439766081871344</v>
+        <v>0.8309047127622978</v>
       </c>
       <c r="C3" t="n">
-        <v>0.7980952380952381</v>
+        <v>0.7676190476190476</v>
       </c>
       <c r="D3" t="n">
-        <v>0.5518954248366013</v>
+        <v>0.6575271512113616</v>
       </c>
     </row>
     <row r="4">
@@ -1254,13 +1254,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.7783969728242173</v>
+        <v>0.7658479532163742</v>
       </c>
       <c r="C4" t="n">
-        <v>0.7199134199134198</v>
+        <v>0.762063492063492</v>
       </c>
       <c r="D4" t="n">
-        <v>0.5445793972109761</v>
+        <v>0.5473684210526316</v>
       </c>
     </row>
     <row r="5">
@@ -1273,7 +1273,7 @@
         <v>0.7823809523809524</v>
       </c>
       <c r="C5" t="n">
-        <v>0.7042857142857143</v>
+        <v>0.7244444444444443</v>
       </c>
       <c r="D5" t="n">
         <v>0.5116939407341883</v>
@@ -1322,13 +1322,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.8777777777777779</v>
+        <v>0.8822222222222222</v>
       </c>
       <c r="C2" t="n">
-        <v>0.77</v>
+        <v>0.75</v>
       </c>
       <c r="D2" t="n">
-        <v>0.5456790123456791</v>
+        <v>0.5530864197530864</v>
       </c>
     </row>
     <row r="3">
@@ -1338,13 +1338,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.9133333333333333</v>
+        <v>0.9066666666666666</v>
       </c>
       <c r="C3" t="n">
-        <v>0.86</v>
+        <v>0.8800000000000001</v>
       </c>
       <c r="D3" t="n">
-        <v>0.6271604938271605</v>
+        <v>0.6814814814814816</v>
       </c>
     </row>
     <row r="4">
@@ -1354,13 +1354,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.8733333333333333</v>
+        <v>0.8666666666666666</v>
       </c>
       <c r="C4" t="n">
-        <v>0.82</v>
+        <v>0.8600000000000001</v>
       </c>
       <c r="D4" t="n">
-        <v>0.6320987654320988</v>
+        <v>0.6419753086419753</v>
       </c>
     </row>
     <row r="5">
@@ -1376,7 +1376,7 @@
         <v>0.8699999999999999</v>
       </c>
       <c r="D5" t="n">
-        <v>0.5950617283950617</v>
+        <v>0.5975308641975309</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Model Improvement: Added Feature Selection (Top 10) and SVM to reduce overfitting
</commit_message>
<xml_diff>
--- a/classification_results/regularized/comprehensive_results.xlsx
+++ b/classification_results/regularized/comprehensive_results.xlsx
@@ -515,40 +515,40 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.7684210526315789</v>
+        <v>0.7714285714285715</v>
       </c>
       <c r="D2" t="n">
-        <v>0.09761703679469162</v>
+        <v>0.09233675918888246</v>
       </c>
       <c r="E2" t="n">
-        <v>0.9447368421052632</v>
+        <v>0.9476190476190476</v>
       </c>
       <c r="F2" t="n">
-        <v>0.1763157894736843</v>
+        <v>0.1761904761904761</v>
       </c>
       <c r="G2" t="n">
-        <v>0.8666666666666666</v>
+        <v>0.8672727272727274</v>
       </c>
       <c r="H2" t="n">
-        <v>0.07027283689263066</v>
+        <v>0.09370253619436458</v>
       </c>
       <c r="I2" t="n">
-        <v>0.7658479532163742</v>
+        <v>0.786969696969697</v>
       </c>
       <c r="J2" t="n">
-        <v>0.09998570398136811</v>
+        <v>0.1030463445622407</v>
       </c>
       <c r="K2" t="n">
-        <v>0.7365656565656564</v>
+        <v>0.7519147519147519</v>
       </c>
       <c r="L2" t="n">
-        <v>0.1008451177889093</v>
+        <v>0.06836878811107963</v>
       </c>
       <c r="M2" t="n">
-        <v>0.7999999999999999</v>
+        <v>0.8363636363636363</v>
       </c>
       <c r="N2" t="n">
-        <v>0.1088662107903635</v>
+        <v>0.1564059139462296</v>
       </c>
     </row>
     <row r="3">
@@ -563,40 +563,40 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.8736842105263157</v>
+        <v>0.8095238095238095</v>
       </c>
       <c r="D3" t="n">
-        <v>0.04210526315789474</v>
+        <v>0.1085881357237274</v>
       </c>
       <c r="E3" t="n">
-        <v>0.8842105263157893</v>
+        <v>0.8904761904761905</v>
       </c>
       <c r="F3" t="n">
-        <v>0.01052631578947361</v>
+        <v>0.080952380952381</v>
       </c>
       <c r="G3" t="n">
-        <v>0.8822222222222222</v>
+        <v>0.8672727272727272</v>
       </c>
       <c r="H3" t="n">
-        <v>0.08680899993166491</v>
+        <v>0.09210127375937413</v>
       </c>
       <c r="I3" t="n">
-        <v>0.8711111111111111</v>
+        <v>0.8122259383128949</v>
       </c>
       <c r="J3" t="n">
-        <v>0.03555555555555552</v>
+        <v>0.1353405936876434</v>
       </c>
       <c r="K3" t="n">
-        <v>0.8565656565656565</v>
+        <v>0.7933699633699633</v>
       </c>
       <c r="L3" t="n">
-        <v>0.06464646464646462</v>
+        <v>0.07381133256584507</v>
       </c>
       <c r="M3" t="n">
-        <v>0.888888888888889</v>
+        <v>0.8545454545454545</v>
       </c>
       <c r="N3" t="n">
-        <v>1.110223024625157e-16</v>
+        <v>0.2040904029149423</v>
       </c>
     </row>
     <row r="4">
@@ -611,40 +611,40 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.8315789473684211</v>
+        <v>0.7999999999999999</v>
       </c>
       <c r="D4" t="n">
-        <v>0.03938586722919937</v>
+        <v>0.1102460657408593</v>
       </c>
       <c r="E4" t="n">
-        <v>0.9921052631578948</v>
+        <v>0.9928571428571429</v>
       </c>
       <c r="F4" t="n">
-        <v>0.1605263157894737</v>
+        <v>0.1928571428571429</v>
       </c>
       <c r="G4" t="n">
-        <v>0.9066666666666666</v>
+        <v>0.8672727272727272</v>
       </c>
       <c r="H4" t="n">
-        <v>0.08508528764034064</v>
+        <v>0.08422716234109436</v>
       </c>
       <c r="I4" t="n">
-        <v>0.8309047127622978</v>
+        <v>0.8020518225735618</v>
       </c>
       <c r="J4" t="n">
-        <v>0.03302185523827871</v>
+        <v>0.1348789604595163</v>
       </c>
       <c r="K4" t="n">
-        <v>0.8036868686868687</v>
+        <v>0.7898268398268399</v>
       </c>
       <c r="L4" t="n">
-        <v>0.06933510216481169</v>
+        <v>0.07526245128566754</v>
       </c>
       <c r="M4" t="n">
-        <v>0.8666666666666666</v>
+        <v>0.8363636363636363</v>
       </c>
       <c r="N4" t="n">
-        <v>0.04444444444444442</v>
+        <v>0.2024641586483645</v>
       </c>
     </row>
     <row r="5">
@@ -659,40 +659,40 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.7789473684210526</v>
+        <v>0.7904761904761906</v>
       </c>
       <c r="D5" t="n">
-        <v>0.06982367979695579</v>
+        <v>0.07737179432986631</v>
       </c>
       <c r="E5" t="n">
-        <v>0.9289473684210525</v>
+        <v>0.9333333333333333</v>
       </c>
       <c r="F5" t="n">
-        <v>0.1499999999999999</v>
+        <v>0.1428571428571428</v>
       </c>
       <c r="G5" t="n">
-        <v>0.8266666666666665</v>
+        <v>0.8654545454545455</v>
       </c>
       <c r="H5" t="n">
-        <v>0.1041366623454221</v>
+        <v>0.1004781954883498</v>
       </c>
       <c r="I5" t="n">
-        <v>0.7823809523809524</v>
+        <v>0.8166329966329966</v>
       </c>
       <c r="J5" t="n">
-        <v>0.06693144697452993</v>
+        <v>0.05502783746501732</v>
       </c>
       <c r="K5" t="n">
-        <v>0.7411255411255412</v>
+        <v>0.7812992562992563</v>
       </c>
       <c r="L5" t="n">
-        <v>0.08498090206193512</v>
+        <v>0.1067447012989573</v>
       </c>
       <c r="M5" t="n">
-        <v>0.8444444444444444</v>
+        <v>0.8727272727272727</v>
       </c>
       <c r="N5" t="n">
-        <v>0.1133115447465063</v>
+        <v>0.07272727272727271</v>
       </c>
     </row>
     <row r="6">
@@ -707,40 +707,40 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.5888888888888889</v>
+        <v>0.5900000000000001</v>
       </c>
       <c r="D6" t="n">
-        <v>0.06666666666666667</v>
+        <v>0.1067707825203131</v>
       </c>
       <c r="E6" t="n">
-        <v>0.9472222222222222</v>
+        <v>0.905</v>
       </c>
       <c r="F6" t="n">
-        <v>0.3583333333333333</v>
+        <v>0.3149999999999999</v>
       </c>
       <c r="G6" t="n">
-        <v>0.6419753086419753</v>
+        <v>0.6383838383838384</v>
       </c>
       <c r="H6" t="n">
-        <v>0.1050471475860871</v>
+        <v>0.1516363151902643</v>
       </c>
       <c r="I6" t="n">
-        <v>0.5473684210526316</v>
+        <v>0.4143503555268261</v>
       </c>
       <c r="J6" t="n">
-        <v>0.1279940493127902</v>
+        <v>0.1762172874458938</v>
       </c>
       <c r="K6" t="n">
-        <v>0.6066666666666667</v>
+        <v>0.575</v>
       </c>
       <c r="L6" t="n">
-        <v>0.06347936380926975</v>
+        <v>0.2529822128134703</v>
       </c>
       <c r="M6" t="n">
-        <v>0.5333333333333334</v>
+        <v>0.3333333333333334</v>
       </c>
       <c r="N6" t="n">
-        <v>0.1777777777777778</v>
+        <v>0.1571348402636772</v>
       </c>
     </row>
     <row r="7">
@@ -755,40 +755,40 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.5777777777777778</v>
+        <v>0.61</v>
       </c>
       <c r="D7" t="n">
-        <v>0.05665577237325316</v>
+        <v>0.1356465996625053</v>
       </c>
       <c r="E7" t="n">
-        <v>0.7583333333333333</v>
+        <v>0.7575</v>
       </c>
       <c r="F7" t="n">
-        <v>0.1805555555555555</v>
+        <v>0.1475</v>
       </c>
       <c r="G7" t="n">
-        <v>0.5530864197530864</v>
+        <v>0.6686868686868687</v>
       </c>
       <c r="H7" t="n">
-        <v>0.07784633466881205</v>
+        <v>0.1561447584560775</v>
       </c>
       <c r="I7" t="n">
-        <v>0.5738588896483632</v>
+        <v>0.512864967849488</v>
       </c>
       <c r="J7" t="n">
-        <v>0.100569593215003</v>
+        <v>0.1659167571900326</v>
       </c>
       <c r="K7" t="n">
-        <v>0.5741880341880343</v>
+        <v>0.6</v>
       </c>
       <c r="L7" t="n">
-        <v>0.04214429294012985</v>
+        <v>0.1837117307087384</v>
       </c>
       <c r="M7" t="n">
-        <v>0.6</v>
+        <v>0.4666666666666667</v>
       </c>
       <c r="N7" t="n">
-        <v>0.180534186769688</v>
+        <v>0.1777777777777778</v>
       </c>
     </row>
     <row r="8">
@@ -803,40 +803,40 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.6555555555555556</v>
+        <v>0.65</v>
       </c>
       <c r="D8" t="n">
-        <v>0.06478835438716998</v>
+        <v>0.130384048104053</v>
       </c>
       <c r="E8" t="n">
-        <v>0.9805555555555555</v>
+        <v>0.9800000000000001</v>
       </c>
       <c r="F8" t="n">
-        <v>0.325</v>
+        <v>0.3300000000000001</v>
       </c>
       <c r="G8" t="n">
-        <v>0.6814814814814816</v>
+        <v>0.7070707070707071</v>
       </c>
       <c r="H8" t="n">
-        <v>0.1068882015896956</v>
+        <v>0.1463775428908024</v>
       </c>
       <c r="I8" t="n">
-        <v>0.6575271512113616</v>
+        <v>0.6026745786033711</v>
       </c>
       <c r="J8" t="n">
-        <v>0.09466974295331763</v>
+        <v>0.1301464626347108</v>
       </c>
       <c r="K8" t="n">
-        <v>0.6450505050505051</v>
+        <v>0.6339682539682541</v>
       </c>
       <c r="L8" t="n">
-        <v>0.04906887313546757</v>
+        <v>0.1584407281878698</v>
       </c>
       <c r="M8" t="n">
-        <v>0.6888888888888889</v>
+        <v>0.5777777777777778</v>
       </c>
       <c r="N8" t="n">
-        <v>0.1632993161855452</v>
+        <v>0.1088662107903635</v>
       </c>
     </row>
     <row r="9">
@@ -851,40 +851,40 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.5444444444444445</v>
+        <v>0.62</v>
       </c>
       <c r="D9" t="n">
-        <v>0.0816496580927726</v>
+        <v>0.1122497216032182</v>
       </c>
       <c r="E9" t="n">
-        <v>0.9555555555555555</v>
+        <v>0.9075000000000001</v>
       </c>
       <c r="F9" t="n">
-        <v>0.411111111111111</v>
+        <v>0.2875000000000001</v>
       </c>
       <c r="G9" t="n">
-        <v>0.5975308641975309</v>
+        <v>0.6363636363636364</v>
       </c>
       <c r="H9" t="n">
-        <v>0.09802189254952696</v>
+        <v>0.1233812645220402</v>
       </c>
       <c r="I9" t="n">
-        <v>0.5116939407341883</v>
+        <v>0.4716526610644258</v>
       </c>
       <c r="J9" t="n">
-        <v>0.1444145070927954</v>
+        <v>0.2010302615297857</v>
       </c>
       <c r="K9" t="n">
-        <v>0.5272727272727272</v>
+        <v>0.6875757575757576</v>
       </c>
       <c r="L9" t="n">
-        <v>0.08351770238440617</v>
+        <v>0.2279271386487329</v>
       </c>
       <c r="M9" t="n">
-        <v>0.5111111111111111</v>
+        <v>0.4222222222222222</v>
       </c>
       <c r="N9" t="n">
-        <v>0.193728841935141</v>
+        <v>0.2154524381073924</v>
       </c>
     </row>
     <row r="10">
@@ -899,40 +899,40 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0.7777777777777778</v>
+        <v>0.7555555555555554</v>
       </c>
       <c r="D10" t="n">
-        <v>0.1571348402636772</v>
+        <v>0.1632993161855452</v>
       </c>
       <c r="E10" t="n">
-        <v>0.9944444444444445</v>
+        <v>0.9777777777777779</v>
       </c>
       <c r="F10" t="n">
-        <v>0.2166666666666667</v>
+        <v>0.2222222222222224</v>
       </c>
       <c r="G10" t="n">
-        <v>0.8600000000000001</v>
+        <v>0.8099999999999999</v>
       </c>
       <c r="H10" t="n">
-        <v>0.1067707825203131</v>
+        <v>0.1019803902718557</v>
       </c>
       <c r="I10" t="n">
-        <v>0.762063492063492</v>
+        <v>0.7354689754689755</v>
       </c>
       <c r="J10" t="n">
-        <v>0.1645905461167204</v>
+        <v>0.1664586421894694</v>
       </c>
       <c r="K10" t="n">
-        <v>0.7833333333333333</v>
+        <v>0.8066666666666666</v>
       </c>
       <c r="L10" t="n">
-        <v>0.19436506316151</v>
+        <v>0.2194943684420577</v>
       </c>
       <c r="M10" t="n">
-        <v>0.76</v>
+        <v>0.71</v>
       </c>
       <c r="N10" t="n">
-        <v>0.1593737745050923</v>
+        <v>0.1907878402833891</v>
       </c>
     </row>
     <row r="11">
@@ -947,40 +947,40 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.6444444444444445</v>
+        <v>0.6888888888888889</v>
       </c>
       <c r="D11" t="n">
-        <v>0.257240820062005</v>
+        <v>0.1777777777777778</v>
       </c>
       <c r="E11" t="n">
-        <v>0.888888888888889</v>
+        <v>0.9166666666666666</v>
       </c>
       <c r="F11" t="n">
-        <v>0.2444444444444445</v>
+        <v>0.2277777777777777</v>
       </c>
       <c r="G11" t="n">
-        <v>0.75</v>
+        <v>0.77</v>
       </c>
       <c r="H11" t="n">
-        <v>0.1949358868961793</v>
+        <v>0.198997487421324</v>
       </c>
       <c r="I11" t="n">
-        <v>0.611111111111111</v>
+        <v>0.67</v>
       </c>
       <c r="J11" t="n">
-        <v>0.2533723166886974</v>
+        <v>0.2111871208194288</v>
       </c>
       <c r="K11" t="n">
         <v>0.6933333333333334</v>
       </c>
       <c r="L11" t="n">
-        <v>0.2969474326842678</v>
+        <v>0.247341419454522</v>
       </c>
       <c r="M11" t="n">
-        <v>0.58</v>
+        <v>0.6799999999999999</v>
       </c>
       <c r="N11" t="n">
-        <v>0.2657066051117284</v>
+        <v>0.2501999200639361</v>
       </c>
     </row>
     <row r="12">
@@ -995,40 +995,40 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0.7777777777777777</v>
+        <v>0.8222222222222222</v>
       </c>
       <c r="D12" t="n">
-        <v>0.1217161238900369</v>
+        <v>0.05443310539518171</v>
       </c>
       <c r="E12" t="n">
-        <v>1</v>
+        <v>0.9944444444444445</v>
       </c>
       <c r="F12" t="n">
-        <v>0.2222222222222223</v>
+        <v>0.1722222222222223</v>
       </c>
       <c r="G12" t="n">
-        <v>0.8800000000000001</v>
+        <v>0.8699999999999999</v>
       </c>
       <c r="H12" t="n">
-        <v>0.08124038404635961</v>
+        <v>0.116619037896906</v>
       </c>
       <c r="I12" t="n">
-        <v>0.7676190476190476</v>
+        <v>0.8025396825396826</v>
       </c>
       <c r="J12" t="n">
-        <v>0.1447619047619048</v>
+        <v>0.07604218372865965</v>
       </c>
       <c r="K12" t="n">
-        <v>0.7466666666666667</v>
+        <v>0.8933333333333333</v>
       </c>
       <c r="L12" t="n">
-        <v>0.1423610433604175</v>
+        <v>0.1372750685464934</v>
       </c>
       <c r="M12" t="n">
-        <v>0.8099999999999999</v>
+        <v>0.77</v>
       </c>
       <c r="N12" t="n">
-        <v>0.1854723699099141</v>
+        <v>0.16</v>
       </c>
     </row>
     <row r="13">
@@ -1046,37 +1046,37 @@
         <v>0.7777777777777777</v>
       </c>
       <c r="D13" t="n">
-        <v>0.1987615979999813</v>
+        <v>0.1217161238900369</v>
       </c>
       <c r="E13" t="n">
-        <v>0.9722222222222223</v>
+        <v>0.9388888888888889</v>
       </c>
       <c r="F13" t="n">
-        <v>0.1944444444444446</v>
+        <v>0.1611111111111112</v>
       </c>
       <c r="G13" t="n">
         <v>0.8699999999999999</v>
       </c>
       <c r="H13" t="n">
-        <v>0.09797958971132713</v>
+        <v>0.1077032961426901</v>
       </c>
       <c r="I13" t="n">
-        <v>0.7244444444444443</v>
+        <v>0.7042857142857143</v>
       </c>
       <c r="J13" t="n">
-        <v>0.2504711609529843</v>
+        <v>0.204420534932381</v>
       </c>
       <c r="K13" t="n">
-        <v>0.8400000000000001</v>
+        <v>0.8433333333333334</v>
       </c>
       <c r="L13" t="n">
-        <v>0.233238075793812</v>
+        <v>0.1348249894410446</v>
       </c>
       <c r="M13" t="n">
-        <v>0.71</v>
+        <v>0.6599999999999999</v>
       </c>
       <c r="N13" t="n">
-        <v>0.2939387691339814</v>
+        <v>0.2596150997149434</v>
       </c>
     </row>
   </sheetData>
@@ -1122,13 +1122,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.8736842105263157</v>
+        <v>0.8095238095238095</v>
       </c>
       <c r="C2" t="n">
-        <v>0.6444444444444445</v>
+        <v>0.6888888888888889</v>
       </c>
       <c r="D2" t="n">
-        <v>0.5777777777777778</v>
+        <v>0.61</v>
       </c>
     </row>
     <row r="3">
@@ -1138,13 +1138,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.8315789473684211</v>
+        <v>0.7999999999999999</v>
       </c>
       <c r="C3" t="n">
-        <v>0.7777777777777777</v>
+        <v>0.8222222222222222</v>
       </c>
       <c r="D3" t="n">
-        <v>0.6555555555555556</v>
+        <v>0.65</v>
       </c>
     </row>
     <row r="4">
@@ -1154,13 +1154,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.7684210526315789</v>
+        <v>0.7714285714285715</v>
       </c>
       <c r="C4" t="n">
-        <v>0.7777777777777778</v>
+        <v>0.7555555555555554</v>
       </c>
       <c r="D4" t="n">
-        <v>0.5888888888888889</v>
+        <v>0.5900000000000001</v>
       </c>
     </row>
     <row r="5">
@@ -1170,13 +1170,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.7789473684210526</v>
+        <v>0.7904761904761906</v>
       </c>
       <c r="C5" t="n">
         <v>0.7777777777777777</v>
       </c>
       <c r="D5" t="n">
-        <v>0.5444444444444445</v>
+        <v>0.62</v>
       </c>
     </row>
   </sheetData>
@@ -1222,13 +1222,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.8711111111111111</v>
+        <v>0.8122259383128949</v>
       </c>
       <c r="C2" t="n">
-        <v>0.611111111111111</v>
+        <v>0.67</v>
       </c>
       <c r="D2" t="n">
-        <v>0.5738588896483632</v>
+        <v>0.512864967849488</v>
       </c>
     </row>
     <row r="3">
@@ -1238,13 +1238,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.8309047127622978</v>
+        <v>0.8020518225735618</v>
       </c>
       <c r="C3" t="n">
-        <v>0.7676190476190476</v>
+        <v>0.8025396825396826</v>
       </c>
       <c r="D3" t="n">
-        <v>0.6575271512113616</v>
+        <v>0.6026745786033711</v>
       </c>
     </row>
     <row r="4">
@@ -1254,13 +1254,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.7658479532163742</v>
+        <v>0.786969696969697</v>
       </c>
       <c r="C4" t="n">
-        <v>0.762063492063492</v>
+        <v>0.7354689754689755</v>
       </c>
       <c r="D4" t="n">
-        <v>0.5473684210526316</v>
+        <v>0.4143503555268261</v>
       </c>
     </row>
     <row r="5">
@@ -1270,13 +1270,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.7823809523809524</v>
+        <v>0.8166329966329966</v>
       </c>
       <c r="C5" t="n">
-        <v>0.7244444444444443</v>
+        <v>0.7042857142857143</v>
       </c>
       <c r="D5" t="n">
-        <v>0.5116939407341883</v>
+        <v>0.4716526610644258</v>
       </c>
     </row>
   </sheetData>
@@ -1322,13 +1322,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.8822222222222222</v>
+        <v>0.8672727272727272</v>
       </c>
       <c r="C2" t="n">
-        <v>0.75</v>
+        <v>0.77</v>
       </c>
       <c r="D2" t="n">
-        <v>0.5530864197530864</v>
+        <v>0.6686868686868687</v>
       </c>
     </row>
     <row r="3">
@@ -1338,13 +1338,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.9066666666666666</v>
+        <v>0.8672727272727272</v>
       </c>
       <c r="C3" t="n">
-        <v>0.8800000000000001</v>
+        <v>0.8699999999999999</v>
       </c>
       <c r="D3" t="n">
-        <v>0.6814814814814816</v>
+        <v>0.7070707070707071</v>
       </c>
     </row>
     <row r="4">
@@ -1354,13 +1354,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.8666666666666666</v>
+        <v>0.8672727272727274</v>
       </c>
       <c r="C4" t="n">
-        <v>0.8600000000000001</v>
+        <v>0.8099999999999999</v>
       </c>
       <c r="D4" t="n">
-        <v>0.6419753086419753</v>
+        <v>0.6383838383838384</v>
       </c>
     </row>
     <row r="5">
@@ -1370,13 +1370,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.8266666666666665</v>
+        <v>0.8654545454545455</v>
       </c>
       <c r="C5" t="n">
         <v>0.8699999999999999</v>
       </c>
       <c r="D5" t="n">
-        <v>0.5975308641975309</v>
+        <v>0.6363636363636364</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Final Polish: Applied Muted/Darker Pastel colors to feature plots and uniform k=15 selection
</commit_message>
<xml_diff>
--- a/classification_results/regularized/comprehensive_results.xlsx
+++ b/classification_results/regularized/comprehensive_results.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N13"/>
+  <dimension ref="A1:N19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -515,40 +515,40 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.7714285714285715</v>
+        <v>0.8095238095238095</v>
       </c>
       <c r="D2" t="n">
-        <v>0.09233675918888246</v>
+        <v>0.09035079029052515</v>
       </c>
       <c r="E2" t="n">
-        <v>0.9476190476190476</v>
+        <v>0.9380952380952381</v>
       </c>
       <c r="F2" t="n">
-        <v>0.1761904761904761</v>
+        <v>0.1285714285714286</v>
       </c>
       <c r="G2" t="n">
-        <v>0.8672727272727274</v>
+        <v>0.8927272727272726</v>
       </c>
       <c r="H2" t="n">
-        <v>0.09370253619436458</v>
+        <v>0.06690316179263309</v>
       </c>
       <c r="I2" t="n">
-        <v>0.786969696969697</v>
+        <v>0.818133971291866</v>
       </c>
       <c r="J2" t="n">
-        <v>0.1030463445622407</v>
+        <v>0.1032903626326882</v>
       </c>
       <c r="K2" t="n">
-        <v>0.7519147519147519</v>
+        <v>0.7977522477522478</v>
       </c>
       <c r="L2" t="n">
-        <v>0.06836878811107963</v>
+        <v>0.07042645291064697</v>
       </c>
       <c r="M2" t="n">
-        <v>0.8363636363636363</v>
+        <v>0.8545454545454547</v>
       </c>
       <c r="N2" t="n">
-        <v>0.1564059139462296</v>
+        <v>0.1585054161287518</v>
       </c>
     </row>
     <row r="3">
@@ -563,40 +563,40 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.8095238095238095</v>
+        <v>0.8285714285714285</v>
       </c>
       <c r="D3" t="n">
-        <v>0.1085881357237274</v>
+        <v>0.04856209060564558</v>
       </c>
       <c r="E3" t="n">
-        <v>0.8904761904761905</v>
+        <v>0.8404761904761905</v>
       </c>
       <c r="F3" t="n">
-        <v>0.080952380952381</v>
+        <v>0.01190476190476197</v>
       </c>
       <c r="G3" t="n">
-        <v>0.8672727272727272</v>
+        <v>0.8618181818181817</v>
       </c>
       <c r="H3" t="n">
-        <v>0.09210127375937413</v>
+        <v>0.06690316179263311</v>
       </c>
       <c r="I3" t="n">
-        <v>0.8122259383128949</v>
+        <v>0.8405122337616616</v>
       </c>
       <c r="J3" t="n">
-        <v>0.1353405936876434</v>
+        <v>0.05911756668454306</v>
       </c>
       <c r="K3" t="n">
-        <v>0.7933699633699633</v>
+        <v>0.8114102564102564</v>
       </c>
       <c r="L3" t="n">
-        <v>0.07381133256584507</v>
+        <v>0.05216609794826454</v>
       </c>
       <c r="M3" t="n">
-        <v>0.8545454545454545</v>
+        <v>0.890909090909091</v>
       </c>
       <c r="N3" t="n">
-        <v>0.2040904029149423</v>
+        <v>0.133608531424537</v>
       </c>
     </row>
     <row r="4">
@@ -607,44 +607,44 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>MLP Classifier</t>
+          <t>SVM</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.7999999999999999</v>
+        <v>0.819047619047619</v>
       </c>
       <c r="D4" t="n">
-        <v>0.1102460657408593</v>
+        <v>0.05553287518900288</v>
       </c>
       <c r="E4" t="n">
-        <v>0.9928571428571429</v>
+        <v>0.8904761904761905</v>
       </c>
       <c r="F4" t="n">
-        <v>0.1928571428571429</v>
+        <v>0.07142857142857151</v>
       </c>
       <c r="G4" t="n">
-        <v>0.8672727272727272</v>
+        <v>0.8818181818181818</v>
       </c>
       <c r="H4" t="n">
-        <v>0.08422716234109436</v>
+        <v>0.08851390141554971</v>
       </c>
       <c r="I4" t="n">
-        <v>0.8020518225735618</v>
+        <v>0.835932523616734</v>
       </c>
       <c r="J4" t="n">
-        <v>0.1348789604595163</v>
+        <v>0.06272874464893786</v>
       </c>
       <c r="K4" t="n">
-        <v>0.7898268398268399</v>
+        <v>0.7908974358974359</v>
       </c>
       <c r="L4" t="n">
-        <v>0.07526245128566754</v>
+        <v>0.06218739261489288</v>
       </c>
       <c r="M4" t="n">
-        <v>0.8363636363636363</v>
+        <v>0.9090909090909092</v>
       </c>
       <c r="N4" t="n">
-        <v>0.2024641586483645</v>
+        <v>0.1408357580439061</v>
       </c>
     </row>
     <row r="5">
@@ -655,140 +655,140 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>MLP Classifier</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.7904761904761906</v>
+        <v>0.8095238095238095</v>
       </c>
       <c r="D5" t="n">
-        <v>0.07737179432986631</v>
+        <v>0.04259177099999599</v>
       </c>
       <c r="E5" t="n">
-        <v>0.9333333333333333</v>
+        <v>0.9071428571428571</v>
       </c>
       <c r="F5" t="n">
-        <v>0.1428571428571428</v>
+        <v>0.09761904761904761</v>
       </c>
       <c r="G5" t="n">
-        <v>0.8654545454545455</v>
+        <v>0.8472727272727273</v>
       </c>
       <c r="H5" t="n">
-        <v>0.1004781954883498</v>
+        <v>0.07679531666161044</v>
       </c>
       <c r="I5" t="n">
-        <v>0.8166329966329966</v>
+        <v>0.8265122337616615</v>
       </c>
       <c r="J5" t="n">
-        <v>0.05502783746501732</v>
+        <v>0.05261924354818757</v>
       </c>
       <c r="K5" t="n">
-        <v>0.7812992562992563</v>
+        <v>0.7883333333333333</v>
       </c>
       <c r="L5" t="n">
-        <v>0.1067447012989573</v>
+        <v>0.06008497384232313</v>
       </c>
       <c r="M5" t="n">
-        <v>0.8727272727272727</v>
+        <v>0.890909090909091</v>
       </c>
       <c r="N5" t="n">
-        <v>0.07272727272727271</v>
+        <v>0.133608531424537</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Treated or Not</t>
+          <t>Diseased or Not</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Random Forest</t>
+          <t>Ensemble Voting</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.5900000000000001</v>
+        <v>0.8285714285714285</v>
       </c>
       <c r="D6" t="n">
-        <v>0.1067707825203131</v>
+        <v>0.04856209060564558</v>
       </c>
       <c r="E6" t="n">
-        <v>0.905</v>
+        <v>0.8928571428571429</v>
       </c>
       <c r="F6" t="n">
-        <v>0.3149999999999999</v>
+        <v>0.06428571428571439</v>
       </c>
       <c r="G6" t="n">
-        <v>0.6383838383838384</v>
+        <v>0.8818181818181818</v>
       </c>
       <c r="H6" t="n">
-        <v>0.1516363151902643</v>
+        <v>0.07883448504974108</v>
       </c>
       <c r="I6" t="n">
-        <v>0.4143503555268261</v>
+        <v>0.8430763363257642</v>
       </c>
       <c r="J6" t="n">
-        <v>0.1762172874458938</v>
+        <v>0.05902855499287542</v>
       </c>
       <c r="K6" t="n">
-        <v>0.575</v>
+        <v>0.8042307692307691</v>
       </c>
       <c r="L6" t="n">
-        <v>0.2529822128134703</v>
+        <v>0.05944018922138926</v>
       </c>
       <c r="M6" t="n">
-        <v>0.3333333333333334</v>
+        <v>0.9090909090909092</v>
       </c>
       <c r="N6" t="n">
-        <v>0.1571348402636772</v>
+        <v>0.1408357580439061</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Treated or Not</t>
+          <t>Diseased or Not</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Logistic Regression</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.61</v>
+        <v>0.8</v>
       </c>
       <c r="D7" t="n">
-        <v>0.1356465996625053</v>
+        <v>0.08192690730516788</v>
       </c>
       <c r="E7" t="n">
-        <v>0.7575</v>
+        <v>0.930952380952381</v>
       </c>
       <c r="F7" t="n">
-        <v>0.1475</v>
+        <v>0.1309523809523809</v>
       </c>
       <c r="G7" t="n">
-        <v>0.6686868686868687</v>
+        <v>0.8790909090909091</v>
       </c>
       <c r="H7" t="n">
-        <v>0.1561447584560775</v>
+        <v>0.09215509743617588</v>
       </c>
       <c r="I7" t="n">
-        <v>0.512864967849488</v>
+        <v>0.8280615680615681</v>
       </c>
       <c r="J7" t="n">
-        <v>0.1659167571900326</v>
+        <v>0.05630567551753038</v>
       </c>
       <c r="K7" t="n">
-        <v>0.6</v>
+        <v>0.7835214785214786</v>
       </c>
       <c r="L7" t="n">
-        <v>0.1837117307087384</v>
+        <v>0.1090520998727956</v>
       </c>
       <c r="M7" t="n">
-        <v>0.4666666666666667</v>
+        <v>0.8909090909090909</v>
       </c>
       <c r="N7" t="n">
-        <v>0.1777777777777778</v>
+        <v>0.03636363636363633</v>
       </c>
     </row>
     <row r="8">
@@ -799,44 +799,44 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>MLP Classifier</t>
+          <t>Random Forest</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.65</v>
+        <v>0.59</v>
       </c>
       <c r="D8" t="n">
-        <v>0.130384048104053</v>
+        <v>0.1356465996625054</v>
       </c>
       <c r="E8" t="n">
-        <v>0.9800000000000001</v>
+        <v>0.875</v>
       </c>
       <c r="F8" t="n">
-        <v>0.3300000000000001</v>
+        <v>0.285</v>
       </c>
       <c r="G8" t="n">
-        <v>0.7070707070707071</v>
+        <v>0.6121212121212121</v>
       </c>
       <c r="H8" t="n">
-        <v>0.1463775428908024</v>
+        <v>0.1825574197589068</v>
       </c>
       <c r="I8" t="n">
-        <v>0.6026745786033711</v>
+        <v>0.4463492063492064</v>
       </c>
       <c r="J8" t="n">
-        <v>0.1301464626347108</v>
+        <v>0.2045449816883505</v>
       </c>
       <c r="K8" t="n">
-        <v>0.6339682539682541</v>
+        <v>0.5644444444444445</v>
       </c>
       <c r="L8" t="n">
-        <v>0.1584407281878698</v>
+        <v>0.2683649624791205</v>
       </c>
       <c r="M8" t="n">
-        <v>0.5777777777777778</v>
+        <v>0.3777777777777778</v>
       </c>
       <c r="N8" t="n">
-        <v>0.1088662107903635</v>
+        <v>0.180534186769688</v>
       </c>
     </row>
     <row r="9">
@@ -847,236 +847,524 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>Logistic Regression</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.62</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="D9" t="n">
-        <v>0.1122497216032182</v>
+        <v>0.1319090595827292</v>
       </c>
       <c r="E9" t="n">
-        <v>0.9075000000000001</v>
+        <v>0.72</v>
       </c>
       <c r="F9" t="n">
-        <v>0.2875000000000001</v>
+        <v>0.1599999999999999</v>
       </c>
       <c r="G9" t="n">
-        <v>0.6363636363636364</v>
+        <v>0.6585858585858586</v>
       </c>
       <c r="H9" t="n">
-        <v>0.1233812645220402</v>
+        <v>0.1630492022139884</v>
       </c>
       <c r="I9" t="n">
-        <v>0.4716526610644258</v>
+        <v>0.4541269841269841</v>
       </c>
       <c r="J9" t="n">
-        <v>0.2010302615297857</v>
+        <v>0.1660444925150576</v>
       </c>
       <c r="K9" t="n">
-        <v>0.6875757575757576</v>
+        <v>0.5436507936507937</v>
       </c>
       <c r="L9" t="n">
-        <v>0.2279271386487329</v>
+        <v>0.1916301026611053</v>
       </c>
       <c r="M9" t="n">
         <v>0.4222222222222222</v>
       </c>
       <c r="N9" t="n">
-        <v>0.2154524381073924</v>
+        <v>0.1777777777777778</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Rescued or Not</t>
+          <t>Treated or Not</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Random Forest</t>
+          <t>SVM</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0.7555555555555554</v>
+        <v>0.65</v>
       </c>
       <c r="D10" t="n">
-        <v>0.1632993161855452</v>
+        <v>0.130384048104053</v>
       </c>
       <c r="E10" t="n">
-        <v>0.9777777777777779</v>
+        <v>0.8325000000000001</v>
       </c>
       <c r="F10" t="n">
-        <v>0.2222222222222224</v>
+        <v>0.1825000000000001</v>
       </c>
       <c r="G10" t="n">
-        <v>0.8099999999999999</v>
+        <v>0.7070707070707071</v>
       </c>
       <c r="H10" t="n">
-        <v>0.1019803902718557</v>
+        <v>0.1562231509428784</v>
       </c>
       <c r="I10" t="n">
-        <v>0.7354689754689755</v>
+        <v>0.5149698340874812</v>
       </c>
       <c r="J10" t="n">
-        <v>0.1664586421894694</v>
+        <v>0.2063565194834397</v>
       </c>
       <c r="K10" t="n">
-        <v>0.8066666666666666</v>
+        <v>0.6583333333333333</v>
       </c>
       <c r="L10" t="n">
-        <v>0.2194943684420577</v>
+        <v>0.1833333333333333</v>
       </c>
       <c r="M10" t="n">
-        <v>0.71</v>
+        <v>0.4444444444444445</v>
       </c>
       <c r="N10" t="n">
-        <v>0.1907878402833891</v>
+        <v>0.210818510677892</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Rescued or Not</t>
+          <t>Treated or Not</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Logistic Regression</t>
+          <t>MLP Classifier</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.6888888888888889</v>
+        <v>0.6599999999999999</v>
       </c>
       <c r="D11" t="n">
-        <v>0.1777777777777778</v>
+        <v>0.1496662954709576</v>
       </c>
       <c r="E11" t="n">
-        <v>0.9166666666666666</v>
+        <v>0.8775000000000001</v>
       </c>
       <c r="F11" t="n">
-        <v>0.2277777777777777</v>
+        <v>0.2175000000000001</v>
       </c>
       <c r="G11" t="n">
-        <v>0.77</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="H11" t="n">
-        <v>0.198997487421324</v>
+        <v>0.1562231509428785</v>
       </c>
       <c r="I11" t="n">
-        <v>0.67</v>
+        <v>0.6000574588809883</v>
       </c>
       <c r="J11" t="n">
-        <v>0.2111871208194288</v>
+        <v>0.1761317718218063</v>
       </c>
       <c r="K11" t="n">
-        <v>0.6933333333333334</v>
+        <v>0.6611111111111111</v>
       </c>
       <c r="L11" t="n">
-        <v>0.247341419454522</v>
+        <v>0.1927705730321941</v>
       </c>
       <c r="M11" t="n">
-        <v>0.6799999999999999</v>
+        <v>0.5777777777777777</v>
       </c>
       <c r="N11" t="n">
-        <v>0.2501999200639361</v>
+        <v>0.1911627837120584</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Rescued or Not</t>
+          <t>Treated or Not</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>MLP Classifier</t>
+          <t>Ensemble Voting</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0.8222222222222222</v>
+        <v>0.6199999999999999</v>
       </c>
       <c r="D12" t="n">
-        <v>0.05443310539518171</v>
+        <v>0.116619037896906</v>
       </c>
       <c r="E12" t="n">
-        <v>0.9944444444444445</v>
+        <v>0.845</v>
       </c>
       <c r="F12" t="n">
-        <v>0.1722222222222223</v>
+        <v>0.2250000000000001</v>
       </c>
       <c r="G12" t="n">
-        <v>0.8699999999999999</v>
+        <v>0.6868686868686869</v>
       </c>
       <c r="H12" t="n">
-        <v>0.116619037896906</v>
+        <v>0.178533746224531</v>
       </c>
       <c r="I12" t="n">
-        <v>0.8025396825396826</v>
+        <v>0.4875859331586886</v>
       </c>
       <c r="J12" t="n">
-        <v>0.07604218372865965</v>
+        <v>0.1763786005724745</v>
       </c>
       <c r="K12" t="n">
-        <v>0.8933333333333333</v>
+        <v>0.6333333333333333</v>
       </c>
       <c r="L12" t="n">
-        <v>0.1372750685464934</v>
+        <v>0.19436506316151</v>
       </c>
       <c r="M12" t="n">
-        <v>0.77</v>
+        <v>0.4222222222222222</v>
       </c>
       <c r="N12" t="n">
-        <v>0.16</v>
+        <v>0.1777777777777778</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>Treated or Not</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>0.6100000000000001</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0.1624807680927192</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0.8724999999999999</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0.2624999999999998</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0.6161616161616161</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0.1704648332099312</v>
+      </c>
+      <c r="I13" t="n">
+        <v>0.4597729618163054</v>
+      </c>
+      <c r="J13" t="n">
+        <v>0.2930643053896195</v>
+      </c>
+      <c r="K13" t="n">
+        <v>0.5166666666666666</v>
+      </c>
+      <c r="L13" t="n">
+        <v>0.3431876713662333</v>
+      </c>
+      <c r="M13" t="n">
+        <v>0.4222222222222222</v>
+      </c>
+      <c r="N13" t="n">
+        <v>0.2666666666666667</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
           <t>Rescued or Not</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Random Forest</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>0.711111111111111</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0.1507184440694504</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0.9555555555555555</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0.2444444444444445</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0.1392838827718412</v>
+      </c>
+      <c r="I14" t="n">
+        <v>0.6603174603174603</v>
+      </c>
+      <c r="J14" t="n">
+        <v>0.1960249982772847</v>
+      </c>
+      <c r="K14" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="L14" t="n">
+        <v>0.2190890230020665</v>
+      </c>
+      <c r="M14" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="N14" t="n">
+        <v>0.215870331449229</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Rescued or Not</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Logistic Regression</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>0.5777777777777777</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0.1911627837120584</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0.1722222222222223</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0.2034698994937581</v>
+      </c>
+      <c r="I15" t="n">
+        <v>0.5541847041847042</v>
+      </c>
+      <c r="J15" t="n">
+        <v>0.1906491627925762</v>
+      </c>
+      <c r="K15" t="n">
+        <v>0.6066666666666667</v>
+      </c>
+      <c r="L15" t="n">
+        <v>0.2602562839459085</v>
+      </c>
+      <c r="M15" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="N15" t="n">
+        <v>0.1777638883463118</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Rescued or Not</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>SVM</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>0.7999999999999999</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0.08314794192830979</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0.9111111111111111</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0.1111111111111112</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0.09695359714832658</v>
+      </c>
+      <c r="I16" t="n">
+        <v>0.7392063492063492</v>
+      </c>
+      <c r="J16" t="n">
+        <v>0.1761744594464523</v>
+      </c>
+      <c r="K16" t="n">
+        <v>0.9099999999999999</v>
+      </c>
+      <c r="L16" t="n">
+        <v>0.1113552872566004</v>
+      </c>
+      <c r="M16" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="N16" t="n">
+        <v>0.2111871208194288</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Rescued or Not</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>MLP Classifier</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>0.6222222222222222</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0.193728841935141</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0.2777777777777778</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0.1772004514666935</v>
+      </c>
+      <c r="I17" t="n">
+        <v>0.5811111111111111</v>
+      </c>
+      <c r="J17" t="n">
+        <v>0.209101546599071</v>
+      </c>
+      <c r="K17" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="L17" t="n">
+        <v>0.2925747767665559</v>
+      </c>
+      <c r="M17" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="N17" t="n">
+        <v>0.1777638883463118</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Rescued or Not</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Ensemble Voting</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>0.7555555555555555</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0.12957670877434</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0.9166666666666667</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0.1611111111111112</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0.8200000000000001</v>
+      </c>
+      <c r="H18" t="n">
+        <v>0.1122497216032182</v>
+      </c>
+      <c r="I18" t="n">
+        <v>0.6892063492063493</v>
+      </c>
+      <c r="J18" t="n">
+        <v>0.1998951602262661</v>
+      </c>
+      <c r="K18" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="L18" t="n">
+        <v>0.1959591794226543</v>
+      </c>
+      <c r="M18" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="N18" t="n">
+        <v>0.215870331449229</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Rescued or Not</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
         <is>
           <t>XGBoost</t>
         </is>
       </c>
-      <c r="C13" t="n">
-        <v>0.7777777777777777</v>
-      </c>
-      <c r="D13" t="n">
-        <v>0.1217161238900369</v>
-      </c>
-      <c r="E13" t="n">
-        <v>0.9388888888888889</v>
-      </c>
-      <c r="F13" t="n">
-        <v>0.1611111111111112</v>
-      </c>
-      <c r="G13" t="n">
-        <v>0.8699999999999999</v>
-      </c>
-      <c r="H13" t="n">
-        <v>0.1077032961426901</v>
-      </c>
-      <c r="I13" t="n">
-        <v>0.7042857142857143</v>
-      </c>
-      <c r="J13" t="n">
-        <v>0.204420534932381</v>
-      </c>
-      <c r="K13" t="n">
-        <v>0.8433333333333334</v>
-      </c>
-      <c r="L13" t="n">
-        <v>0.1348249894410446</v>
-      </c>
-      <c r="M13" t="n">
-        <v>0.6599999999999999</v>
-      </c>
-      <c r="N13" t="n">
-        <v>0.2596150997149434</v>
+      <c r="C19" t="n">
+        <v>0.7555555555555555</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0.12957670877434</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0.9166666666666666</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0.1611111111111111</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0.8899999999999999</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0.1113552872566004</v>
+      </c>
+      <c r="I19" t="n">
+        <v>0.6955555555555556</v>
+      </c>
+      <c r="J19" t="n">
+        <v>0.2055525525306165</v>
+      </c>
+      <c r="K19" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="L19" t="n">
+        <v>0.1833030277982336</v>
+      </c>
+      <c r="M19" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="N19" t="n">
+        <v>0.2638181191654584</v>
       </c>
     </row>
   </sheetData>
@@ -1090,7 +1378,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1118,65 +1406,97 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Logistic Regression</t>
+          <t>Ensemble Voting</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.8095238095238095</v>
+        <v>0.8285714285714285</v>
       </c>
       <c r="C2" t="n">
-        <v>0.6888888888888889</v>
+        <v>0.7555555555555555</v>
       </c>
       <c r="D2" t="n">
-        <v>0.61</v>
+        <v>0.6199999999999999</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>MLP Classifier</t>
+          <t>Logistic Regression</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.7999999999999999</v>
+        <v>0.8285714285714285</v>
       </c>
       <c r="C3" t="n">
-        <v>0.8222222222222222</v>
+        <v>0.5777777777777777</v>
       </c>
       <c r="D3" t="n">
-        <v>0.65</v>
+        <v>0.5600000000000001</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>Random Forest</t>
+          <t>MLP Classifier</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.7714285714285715</v>
+        <v>0.8095238095238095</v>
       </c>
       <c r="C4" t="n">
-        <v>0.7555555555555554</v>
+        <v>0.6222222222222222</v>
       </c>
       <c r="D4" t="n">
-        <v>0.5900000000000001</v>
+        <v>0.6599999999999999</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
+          <t>Random Forest</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0.8095238095238095</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0.711111111111111</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.59</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>SVM</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0.819047619047619</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0.7999999999999999</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.65</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
           <t>XGBoost</t>
         </is>
       </c>
-      <c r="B5" t="n">
-        <v>0.7904761904761906</v>
-      </c>
-      <c r="C5" t="n">
-        <v>0.7777777777777777</v>
-      </c>
-      <c r="D5" t="n">
-        <v>0.62</v>
+      <c r="B7" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0.7555555555555555</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.6100000000000001</v>
       </c>
     </row>
   </sheetData>
@@ -1190,7 +1510,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1218,65 +1538,97 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Logistic Regression</t>
+          <t>Ensemble Voting</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.8122259383128949</v>
+        <v>0.8430763363257642</v>
       </c>
       <c r="C2" t="n">
-        <v>0.67</v>
+        <v>0.6892063492063493</v>
       </c>
       <c r="D2" t="n">
-        <v>0.512864967849488</v>
+        <v>0.4875859331586886</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>MLP Classifier</t>
+          <t>Logistic Regression</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.8020518225735618</v>
+        <v>0.8405122337616616</v>
       </c>
       <c r="C3" t="n">
-        <v>0.8025396825396826</v>
+        <v>0.5541847041847042</v>
       </c>
       <c r="D3" t="n">
-        <v>0.6026745786033711</v>
+        <v>0.4541269841269841</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>Random Forest</t>
+          <t>MLP Classifier</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.786969696969697</v>
+        <v>0.8265122337616615</v>
       </c>
       <c r="C4" t="n">
-        <v>0.7354689754689755</v>
+        <v>0.5811111111111111</v>
       </c>
       <c r="D4" t="n">
-        <v>0.4143503555268261</v>
+        <v>0.6000574588809883</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
+          <t>Random Forest</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0.818133971291866</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0.6603174603174603</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.4463492063492064</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>SVM</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0.835932523616734</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0.7392063492063492</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.5149698340874812</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
           <t>XGBoost</t>
         </is>
       </c>
-      <c r="B5" t="n">
-        <v>0.8166329966329966</v>
-      </c>
-      <c r="C5" t="n">
-        <v>0.7042857142857143</v>
-      </c>
-      <c r="D5" t="n">
-        <v>0.4716526610644258</v>
+      <c r="B7" t="n">
+        <v>0.8280615680615681</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0.6955555555555556</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.4597729618163054</v>
       </c>
     </row>
   </sheetData>
@@ -1290,7 +1642,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1318,65 +1670,97 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Logistic Regression</t>
+          <t>Ensemble Voting</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.8672727272727272</v>
+        <v>0.8818181818181818</v>
       </c>
       <c r="C2" t="n">
-        <v>0.77</v>
+        <v>0.8200000000000001</v>
       </c>
       <c r="D2" t="n">
-        <v>0.6686868686868687</v>
+        <v>0.6868686868686869</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>MLP Classifier</t>
+          <t>Logistic Regression</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.8672727272727272</v>
+        <v>0.8618181818181817</v>
       </c>
       <c r="C3" t="n">
-        <v>0.8699999999999999</v>
+        <v>0.74</v>
       </c>
       <c r="D3" t="n">
-        <v>0.7070707070707071</v>
+        <v>0.6585858585858586</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>Random Forest</t>
+          <t>MLP Classifier</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.8672727272727274</v>
+        <v>0.8472727272727273</v>
       </c>
       <c r="C4" t="n">
-        <v>0.8099999999999999</v>
+        <v>0.76</v>
       </c>
       <c r="D4" t="n">
-        <v>0.6383838383838384</v>
+        <v>0.6666666666666666</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
+          <t>Random Forest</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0.8927272727272726</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.6121212121212121</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>SVM</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0.8818181818181818</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.7070707070707071</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
           <t>XGBoost</t>
         </is>
       </c>
-      <c r="B5" t="n">
-        <v>0.8654545454545455</v>
-      </c>
-      <c r="C5" t="n">
-        <v>0.8699999999999999</v>
-      </c>
-      <c r="D5" t="n">
-        <v>0.6363636363636364</v>
+      <c r="B7" t="n">
+        <v>0.8790909090909091</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0.8899999999999999</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.6161616161616161</v>
       </c>
     </row>
   </sheetData>

</xml_diff>